<commit_message>
Stage 2: collectors for 19 sources, registry v0.4 updates
- collectors/: common RawEvent format and Collector interface, polite HTTP client
  (robots.txt, per-host delay / Crawl-delay, 429 back-off, optional curl backend),
  iCal / JSON-LD / RSS parsers, one module per source
- scripts/run_collectors.py: runs collectors, writes data/raw/<ID>_<module>.json
- scripts/stage2_report.py: per-source counts, field fill rates, control events
- Registry v0.4: Eventbrite to P1, new S090 DesignMyNight (robots.txt disallows events)
  and S091 Cambridge Live Tickets, stage-1 decisions, 5 talks.cam lists,
  'Контрольные события' sheet from data/control_events.json (+ Oktoberfest)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CLyvgaEdz1GH7PAyWSk6om
</commit_message>
<xml_diff>
--- a/data/cambridge_event_sources_v0.4.xlsx
+++ b/data/cambridge_event_sources_v0.4.xlsx
@@ -10,13 +10,14 @@
     <sheet name="Как пользоваться" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Источники" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Проверка P1" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Сводка" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Схема события" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Категории и теги" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Контрольные события" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Сводка" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Схема события" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Категории и теги" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Источники'!$A$1:$O$90</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Проверка P1'!$A$1:$G$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Источники'!$A$1:$O$92</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Проверка P1'!$A$1:$G$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
@@ -80,7 +81,7 @@
       <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -107,6 +108,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF4CCCC"/>
       </patternFill>
     </fill>
     <fill>
@@ -143,7 +149,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -199,14 +205,18 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -507,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="120" customWidth="1" style="10" min="1" max="1"/>
@@ -593,6 +603,13 @@
       <c r="A13" t="inlineStr">
         <is>
           <t>v0.4 (2026-09-27): проверены источники приоритета 1 — см. лист «Проверка P1»; новые столбцы «Endpoint для сбора», «robots.txt», «Проверено». «URL проверен = нет» — URL не отвечает (красный).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>v0.4, правки после этапа 1: Eventbrite (S008) поднят до приоритета 1; добавлены S090 DesignMyNight и S091 Cambridge Live Tickets; лист «Контрольные события» (источник — data/control_events.json).</t>
         </is>
       </c>
     </row>
@@ -609,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O90"/>
+  <dimension ref="A1:O92"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="10" min="1" max="1"/>
@@ -1137,7 +1154,7 @@
       </c>
       <c r="L7" s="16" t="inlineStr">
         <is>
-          <t>Удобно ловить объявления новых шоу</t>
+          <t>Удобно ловить объявления новых шоу. v0.4: JSON-LD на первой странице списка (~37 событий), продолжение подгружается JS; через Ents24 ловим и Arts Theatre (S041)</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1194,7 +1211,7 @@
       </c>
       <c r="H8" s="16" t="inlineStr">
         <is>
-          <t>JSON-LD (API — по ключу)</t>
+          <t>JSON-LD</t>
         </is>
       </c>
       <c r="I8" s="16" t="inlineStr">
@@ -1212,7 +1229,7 @@
       </c>
       <c r="L8" s="16" t="inlineStr">
         <is>
-          <t>Есть API и партнёрка — сразу и данные, и монетизация. v0.4: страница отдаёт ~49 событий JSON-LD; официальный API требует партнёрский ключ (github.com/Skiddle/web-api)</t>
+          <t>Есть API и партнёрка — сразу и данные, и монетизация. v0.4: ~49 событий JSON-LD на первой странице списка; продолжение подгружается JS; API и ключ не нужны (решение после этапа 1)</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1254,7 +1271,7 @@
       </c>
       <c r="E9" s="16" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.co.uk</t>
+          <t>https://www.eventbrite.co.uk/d/united-kingdom--cambridge/all-events/</t>
         </is>
       </c>
       <c r="F9" s="16" t="inlineStr">
@@ -1269,7 +1286,7 @@
       </c>
       <c r="H9" s="16" t="inlineStr">
         <is>
-          <t>HTML (публичный поиск по API закрыт — проверить)</t>
+          <t>JSON-LD</t>
         </is>
       </c>
       <c r="I9" s="16" t="inlineStr">
@@ -1278,16 +1295,31 @@
         </is>
       </c>
       <c r="J9" s="16" t="n">
-        <v>2</v>
-      </c>
-      <c r="K9" s="17" t="inlineStr">
-        <is>
-          <t>проверить</t>
+        <v>1</v>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>да</t>
         </is>
       </c>
       <c r="L9" s="16" t="inlineStr">
         <is>
-          <t>Много шума — нужен жёсткий фильтр</t>
+          <t>Много шума — нужен жёсткий фильтр. v0.4: поднят до P1 в v0.4; 20 событий JSON-LD на страницу, с postcode и координатами; фильтр — почтовые области CB, PE, SG, CM, IP, онлайн отбрасываем</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.co.uk/d/united-kingdom--cambridge/all-events/?page=N</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>разрешено</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
         </is>
       </c>
     </row>
@@ -2595,7 +2627,7 @@
       </c>
       <c r="H31" s="16" t="inlineStr">
         <is>
-          <t>HTML</t>
+          <t>HTML (curl, пауза 10 с)</t>
         </is>
       </c>
       <c r="I31" s="16" t="inlineStr">
@@ -2613,7 +2645,7 @@
       </c>
       <c r="L31" s="16" t="inlineStr">
         <is>
-          <t>v0.4: фестиваль в марте; часть событий дублируется в talks.cam</t>
+          <t>v0.4: решение после этапа 1: собирать через curl с честным User-Agent и паузой 10 с (robots.txt разрешает, Crawl-delay 10); под браузер не маскироваться; фестиваль в марте</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -3309,7 +3341,7 @@
       </c>
       <c r="H42" s="16" t="inlineStr">
         <is>
-          <t>HTML (блок Cloudflare)</t>
+          <t>Через Ents24 (S006)</t>
         </is>
       </c>
       <c r="I42" s="16" t="inlineStr">
@@ -3327,7 +3359,7 @@
       </c>
       <c r="L42" s="16" t="inlineStr">
         <is>
-          <t>v0.4: домен сменился: cambridgeartstheatre.com → artstheatre.co.uk; сайт закрыт для ботов — брать через агрегаторы (Ents24, Visit Cambridge) или спросить разрешения</t>
+          <t>v0.4: решение после этапа 1: защиту не обходим; афишу Arts Theatre берём из Ents24. Домен: cambridgeartstheatre.com → artstheatre.co.uk</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -3699,12 +3731,12 @@
       </c>
       <c r="L48" s="16" t="inlineStr">
         <is>
-          <t>Лучший технический источник: готовые фиды с датой, местом и организатором. v0.4: фиды есть у каждого списка: /show/ics|rss|xml/&lt;id&gt;; список 109 не существует, взят 5606 «Featured talks»; подбор тематических списков — этап 2</t>
+          <t>Лучший технический источник: готовые фиды с датой, местом и организатором. v0.4: 5 публичных списков: 5606 Featured talks, 5462 Major Public Lectures in Cambridge, 5358 Darwin College Lecture Series, 5769 Cabinet of Natural History, 23088 CamTalks; список Fitzwilliam (12614) пуст; фиды /show/ics|rss|xml/&lt;id&gt;</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>https://talks.cam.ac.uk/show/ics/5606/</t>
+          <t>https://talks.cam.ac.uk/show/ics/{5606,5462,5358,5769,23088}/</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -3774,7 +3806,7 @@
       </c>
       <c r="L49" s="16" t="inlineStr">
         <is>
-          <t>v0.4: страница даёт webcal-подписку, но хост фидов запрещает роботов в robots.txt — нужно решение: HTML или запрос разрешения</t>
+          <t>v0.4: решение после этапа 1: уважаем Disallow на webservices.admin.cam.ac.uk; собираем HTML-страницу admin.cam.ac.uk/whatson/ (robots.txt её разрешает); лекции также покрывает talks.cam</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
@@ -4780,7 +4812,7 @@
       </c>
       <c r="H66" s="16" t="inlineStr">
         <is>
-          <t>HTML</t>
+          <t>HTML (curl, пауза 10 с)</t>
         </is>
       </c>
       <c r="I66" s="16" t="inlineStr">
@@ -4798,7 +4830,7 @@
       </c>
       <c r="L66" s="16" t="inlineStr">
         <is>
-          <t>Часть Heritage Open Days. v0.4: ежегодно (сентябрь), часть Heritage Open Days</t>
+          <t>Часть Heritage Open Days. v0.4: решение после этапа 1: curl с честным User-Agent и паузой 10 с; ежегодно (сентябрь), часть Heritage Open Days</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
@@ -5086,7 +5118,7 @@
       </c>
       <c r="H71" s="16" t="inlineStr">
         <is>
-          <t>HTML</t>
+          <t>Ручной сезонный</t>
         </is>
       </c>
       <c r="I71" s="16" t="inlineStr">
@@ -5104,7 +5136,7 @@
       </c>
       <c r="L71" s="16" t="inlineStr">
         <is>
-          <t>v0.4: Wimpole и Anglesey Abbey — HTML живые; сайт защищён Radware — собирать редко или вручную</t>
+          <t>v0.4: решение после этапа 1: защиту Radware не обходим; вносить вручную по сезонам (Wimpole, Anglesey Abbey, Wicken Fen)</t>
         </is>
       </c>
       <c r="M71" t="inlineStr">
@@ -6229,7 +6261,7 @@
       </c>
       <c r="H90" s="16" t="inlineStr">
         <is>
-          <t>Ручной (сайт закрыт для ботов)</t>
+          <t>Через Cambridge News (S004) и Cambridge 105 (S005)</t>
         </is>
       </c>
       <c r="I90" s="16" t="inlineStr">
@@ -6247,7 +6279,7 @@
       </c>
       <c r="L90" s="16" t="inlineStr">
         <is>
-          <t>Нужен и для рубрики «Практическое» — перекрытия. v0.4: официальный сайт найден (MDUK, Bidwells Cambridge 10k); ловить через Cambridge News / Cambridge 105 или вносить вручную раз в год</t>
+          <t>Нужен и для рубрики «Практическое» — перекрытия. v0.4: решение после этапа 1: защиту не обходим; ловим по новостям Cambridge News и Cambridge 105, официальный сайт townandgown10k.com (MDUK)</t>
         </is>
       </c>
       <c r="N90" t="inlineStr">
@@ -6261,8 +6293,158 @@
         </is>
       </c>
     </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>S090</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Ночная жизнь</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>DesignMyNight — Cambridge</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Агрегатор / бронирование</t>
+        </is>
+      </c>
+      <c r="E91" s="19" t="inlineStr">
+        <is>
+          <t>https://www.designmynight.com/cambridge</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Бары, рестораны, мероприятия в заведениях</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Центр</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>— (robots.txt запрещает)</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Еженедельно</t>
+        </is>
+      </c>
+      <c r="J91" t="n">
+        <v>1</v>
+      </c>
+      <c r="K91" s="19" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>Добавлен в v0.4 (решение после этапа 1). v0.4: не собираем; возможен только как справочник заведений для «новое в городе»</t>
+        </is>
+      </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>https://www.designmynight.com/cambridge</t>
+        </is>
+      </c>
+      <c r="N91" t="inlineStr">
+        <is>
+          <t>запрещено: /cambridge/whats-on, /api/</t>
+        </is>
+      </c>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>S091</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Сквозные агрегаторы</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Cambridge Live Tickets</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Билетная система</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>https://www.cambridgelivetickets.co.uk</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Corn Exchange, Guildhall, городские события Cambridge Live</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Центр</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>HTML + JSON-LD</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Ежедневно</t>
+        </is>
+      </c>
+      <c r="J92" t="n">
+        <v>1</v>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>Добавлен в v0.4 (решение после этапа 1). v0.4: список ?page=1..4 в HTML (~24 на страницу), JSON-LD Event с postcode на странице события; пересекается с S011 и S072</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>https://www.cambridgelivetickets.co.uk/events</t>
+        </is>
+      </c>
+      <c r="N92" t="inlineStr">
+        <is>
+          <t>разрешено</t>
+        </is>
+      </c>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O90"/>
+  <autoFilter ref="A1:O92"/>
   <dataValidations count="3">
     <dataValidation sqref="J2:J500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"1,2,3"</formula1>
@@ -6289,7 +6471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="11" min="1" max="1"/>
@@ -6302,69 +6484,69 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="19" t="inlineStr">
+      <c r="A1" s="20" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B1" s="19" t="inlineStr">
+      <c r="B1" s="20" t="inlineStr">
         <is>
           <t>Источник</t>
         </is>
       </c>
-      <c r="C1" s="19" t="inlineStr">
+      <c r="C1" s="20" t="inlineStr">
         <is>
           <t>URL проверен</t>
         </is>
       </c>
-      <c r="D1" s="19" t="inlineStr">
+      <c r="D1" s="20" t="inlineStr">
         <is>
           <t>Способ сбора</t>
         </is>
       </c>
-      <c r="E1" s="19" t="inlineStr">
+      <c r="E1" s="20" t="inlineStr">
         <is>
           <t>Endpoint</t>
         </is>
       </c>
-      <c r="F1" s="19" t="inlineStr">
+      <c r="F1" s="20" t="inlineStr">
         <is>
           <t>Что нашёл</t>
         </is>
       </c>
-      <c r="G1" s="19" t="inlineStr">
+      <c r="G1" s="20" t="inlineStr">
         <is>
           <t>Что не получилось</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="20" t="inlineStr">
+      <c r="A2" s="21" t="inlineStr">
         <is>
           <t>S001</t>
         </is>
       </c>
-      <c r="B2" s="20" t="inlineStr">
+      <c r="B2" s="21" t="inlineStr">
         <is>
           <t>Visit Cambridge — events</t>
         </is>
       </c>
-      <c r="C2" s="21" t="inlineStr">
+      <c r="C2" s="22" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D2" s="20" t="inlineStr">
+      <c r="D2" s="21" t="inlineStr">
         <is>
           <t>API + HTML</t>
         </is>
       </c>
-      <c r="E2" s="20" t="inlineStr">
+      <c r="E2" s="21" t="inlineStr">
         <is>
           <t>https://www.visitcambridge.org/wp-json/vc-map/v1/events</t>
         </is>
       </c>
-      <c r="F2" s="20" t="inlineStr">
+      <c r="F2" s="21" t="inlineStr">
         <is>
           <t>https://www.visitcambridge.org — 200; alternate-фиды: https://www.visitcambridge.org/wp-json/wp/v2/pages/26, https://www.visitcambridge.org/wp-json/oembed/1.0/embed?url=https%3A%2F%2Fwww.visitcambridge.org%2F; WordPress
 https://www.visitcambridge.org/whats-on/ — 200; alternate-фиды: https://www.visitcambridge.org/wp-json/wp/v2/pages/553, https://www.visitcambridge.org/wp-json/oembed/1.0/embed?url=https%3A%2F%2Fwww.visitcambridge.org%2Fwhats-on%2F; WordPress
@@ -6372,107 +6554,107 @@
 https://www.visitcambridge.org/wp-json/vc-map/v1/events — 200; JSON</t>
         </is>
       </c>
-      <c r="G2" s="20" t="inlineStr"/>
+      <c r="G2" s="21" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="20" t="inlineStr">
+      <c r="A3" s="21" t="inlineStr">
         <is>
           <t>S002</t>
         </is>
       </c>
-      <c r="B3" s="20" t="inlineStr">
+      <c r="B3" s="21" t="inlineStr">
         <is>
           <t>What's On In Cambridge</t>
         </is>
       </c>
-      <c r="C3" s="21" t="inlineStr">
+      <c r="C3" s="22" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D3" s="20" t="inlineStr">
+      <c r="D3" s="21" t="inlineStr">
         <is>
           <t>RSS</t>
         </is>
       </c>
-      <c r="E3" s="20" t="inlineStr">
+      <c r="E3" s="21" t="inlineStr">
         <is>
           <t>https://www.whatsonincambridge.com/feed/</t>
         </is>
       </c>
-      <c r="F3" s="20" t="inlineStr">
+      <c r="F3" s="21" t="inlineStr">
         <is>
           <t>https://www.whatsonincambridge.com/__superjs/challenge?u=%2Fevents%2F — 200
 https://www.whatsonincambridge.com/feed/ — 200; фид, записей: 10</t>
         </is>
       </c>
-      <c r="G3" s="20" t="inlineStr">
+      <c r="G3" s="21" t="inlineStr">
         <is>
           <t>https://www.whatsonincambridge.com/events/ — JS-проверка «SuperJS» (бот-блок), HTML без браузера недоступен</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="20" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>S003</t>
         </is>
       </c>
-      <c r="B4" s="20" t="inlineStr">
+      <c r="B4" s="21" t="inlineStr">
         <is>
           <t>Cambridge Independent — What's On</t>
         </is>
       </c>
-      <c r="C4" s="21" t="inlineStr">
+      <c r="C4" s="22" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D4" s="20" t="inlineStr">
+      <c r="D4" s="21" t="inlineStr">
         <is>
           <t>RSS</t>
         </is>
       </c>
-      <c r="E4" s="20" t="inlineStr">
+      <c r="E4" s="21" t="inlineStr">
         <is>
           <t>https://www.cambridgeindependent.co.uk/_api/rss/cambridge_independent_whatson_feed.xml</t>
         </is>
       </c>
-      <c r="F4" s="20" t="inlineStr">
+      <c r="F4" s="21" t="inlineStr">
         <is>
           <t>https://www.cambridgeindependent.co.uk/whats-on/ — 200
 https://www.cambridgeindependent.co.uk/_api/rss/cambridge_independent_whatson_feed.xml — 200; фид, записей: 20</t>
         </is>
       </c>
-      <c r="G4" s="20" t="inlineStr"/>
+      <c r="G4" s="21" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="20" t="inlineStr">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>S004</t>
         </is>
       </c>
-      <c r="B5" s="20" t="inlineStr">
+      <c r="B5" s="21" t="inlineStr">
         <is>
           <t>Cambridge News / CambridgeshireLive</t>
         </is>
       </c>
-      <c r="C5" s="21" t="inlineStr">
+      <c r="C5" s="22" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D5" s="20" t="inlineStr">
+      <c r="D5" s="21" t="inlineStr">
         <is>
           <t>RSS</t>
         </is>
       </c>
-      <c r="E5" s="20" t="inlineStr">
+      <c r="E5" s="21" t="inlineStr">
         <is>
           <t>https://www.cambridge-news.co.uk/whats-on/?service=rss</t>
         </is>
       </c>
-      <c r="F5" s="20" t="inlineStr">
+      <c r="F5" s="21" t="inlineStr">
         <is>
           <t>https://www.cambridge-news.co.uk — 200; alternate-фиды: https://www.cambridge-news.co.uk/rss.xml
 https://www.cambridge-news.co.uk/whats-on/ — 200; alternate-фиды: https://www.cambridge-news.co.uk/whats-on/rss.xml; билетная система: ecal
@@ -6481,35 +6663,35 @@
 https://www.cambridge-news.co.uk/whats-on/?service=rss — 200; фид, записей: 15</t>
         </is>
       </c>
-      <c r="G5" s="20" t="inlineStr"/>
+      <c r="G5" s="21" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="20" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>S005</t>
         </is>
       </c>
-      <c r="B6" s="20" t="inlineStr">
+      <c r="B6" s="21" t="inlineStr">
         <is>
           <t>Cambridge 105 — события</t>
         </is>
       </c>
-      <c r="C6" s="21" t="inlineStr">
+      <c r="C6" s="22" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D6" s="20" t="inlineStr">
+      <c r="D6" s="21" t="inlineStr">
         <is>
           <t>iCal</t>
         </is>
       </c>
-      <c r="E6" s="20" t="inlineStr">
+      <c r="E6" s="21" t="inlineStr">
         <is>
           <t>https://cambridge105.co.uk/whatson/?ical=1</t>
         </is>
       </c>
-      <c r="F6" s="20" t="inlineStr">
+      <c r="F6" s="21" t="inlineStr">
         <is>
           <t>https://cambridge105.co.uk — 200; alternate-фиды: https://cambridge105.co.uk/whatson/?ical=1, https://cambridge105.co.uk/wp-json/wp/v2/pages/44141, https://cambridge105.co.uk/wp-json/oembed/1.0/embed?url=https%3A%2F%2Fcambridge105.co.uk%2F; WordPress
 https://cambridge105.co.uk/events/ — 200; alternate-фиды: https://cambridge105.co.uk/whatson/?ical=1, https://cambridge105.co.uk/wp-json/wp/v2/media/75261, https://cambridge105.co.uk/wp-json/oembed/1.0/embed?url=https%3A%2F%2Fcambridge105.co.uk%2Fevents%2F; WordPress
@@ -6519,102 +6701,136 @@
 https://cambridge105.co.uk/whatson/?ical=1 — 200; iCal, событий: 22</t>
         </is>
       </c>
-      <c r="G6" s="20" t="inlineStr"/>
+      <c r="G6" s="21" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="20" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>S006</t>
         </is>
       </c>
-      <c r="B7" s="20" t="inlineStr">
+      <c r="B7" s="21" t="inlineStr">
         <is>
           <t>Ents24 — Cambridge</t>
         </is>
       </c>
-      <c r="C7" s="21" t="inlineStr">
+      <c r="C7" s="22" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D7" s="20" t="inlineStr">
+      <c r="D7" s="21" t="inlineStr">
         <is>
           <t>JSON-LD</t>
         </is>
       </c>
-      <c r="E7" s="20" t="inlineStr">
+      <c r="E7" s="21" t="inlineStr">
         <is>
           <t>https://www.ents24.com/whatson/cambridge</t>
         </is>
       </c>
-      <c r="F7" s="20" t="inlineStr">
+      <c r="F7" s="21" t="inlineStr">
         <is>
           <t>https://www.ents24.com/whatson/cambridge — 200; JSON-LD Event: 37; билетная система: ents24, gigantic</t>
         </is>
       </c>
-      <c r="G7" s="20" t="inlineStr"/>
+      <c r="G7" s="21" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="20" t="inlineStr">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>S007</t>
         </is>
       </c>
-      <c r="B8" s="20" t="inlineStr">
+      <c r="B8" s="21" t="inlineStr">
         <is>
           <t>Skiddle — Cambridge</t>
         </is>
       </c>
-      <c r="C8" s="21" t="inlineStr">
+      <c r="C8" s="22" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D8" s="20" t="inlineStr">
-        <is>
-          <t>JSON-LD (API — по ключу)</t>
-        </is>
-      </c>
-      <c r="E8" s="20" t="inlineStr">
+      <c r="D8" s="21" t="inlineStr">
+        <is>
+          <t>JSON-LD</t>
+        </is>
+      </c>
+      <c r="E8" s="21" t="inlineStr">
         <is>
           <t>https://www.skiddle.com/whats-on/Cambridge/</t>
         </is>
       </c>
-      <c r="F8" s="20" t="inlineStr">
+      <c r="F8" s="21" t="inlineStr">
         <is>
           <t>https://www.skiddle.com/whats-on/Cambridge/ — 200; JSON-LD Event: 49; билетная система: ecal, skiddle
 https://www.skiddle.com/api/ — 200; билетная система: skiddle</t>
         </is>
       </c>
-      <c r="G8" s="20" t="inlineStr"/>
+      <c r="G8" s="21" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="20" t="inlineStr">
+      <c r="A9" s="21" t="inlineStr">
+        <is>
+          <t>S008</t>
+        </is>
+      </c>
+      <c r="B9" s="21" t="inlineStr">
+        <is>
+          <t>Eventbrite — Cambridge</t>
+        </is>
+      </c>
+      <c r="C9" s="22" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="D9" s="21" t="inlineStr">
+        <is>
+          <t>JSON-LD</t>
+        </is>
+      </c>
+      <c r="E9" s="21" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.co.uk/d/united-kingdom--cambridge/all-events/?page=N</t>
+        </is>
+      </c>
+      <c r="F9" s="21" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.co.uk — 200; билетная система: eventbrite
+https://www.eventbrite.co.uk/d/united-kingdom--cambridge/all-events/ — 200; JSON-LD Event: 20; билетная система: eventbrite</t>
+        </is>
+      </c>
+      <c r="G9" s="21" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="21" t="inlineStr">
         <is>
           <t>S011</t>
         </is>
       </c>
-      <c r="B9" s="20" t="inlineStr">
+      <c r="B10" s="21" t="inlineStr">
         <is>
           <t>Cambridge Corn Exchange</t>
         </is>
       </c>
-      <c r="C9" s="21" t="inlineStr">
+      <c r="C10" s="22" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D9" s="20" t="inlineStr">
+      <c r="D10" s="21" t="inlineStr">
         <is>
           <t>HTML + JSON-LD</t>
         </is>
       </c>
-      <c r="E9" s="20" t="inlineStr">
+      <c r="E10" s="21" t="inlineStr">
         <is>
           <t>https://www.cornex.co.uk/events</t>
         </is>
       </c>
-      <c r="F9" s="20" t="inlineStr">
+      <c r="F10" s="21" t="inlineStr">
         <is>
           <t>https://www.cambridgelivetickets.co.uk/ — 200
 https://www.cornex.co.uk — 200
@@ -6623,35 +6839,35 @@
 https://www.cornex.co.uk/events/alison-moyet-2 — 200; JSON-LD Event: 1</t>
         </is>
       </c>
-      <c r="G9" s="20" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="20" t="inlineStr">
+      <c r="G10" s="21" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>S012</t>
         </is>
       </c>
-      <c r="B10" s="20" t="inlineStr">
+      <c r="B11" s="21" t="inlineStr">
         <is>
           <t>Cambridge Junction</t>
         </is>
       </c>
-      <c r="C10" s="21" t="inlineStr">
+      <c r="C11" s="22" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D10" s="20" t="inlineStr">
+      <c r="D11" s="21" t="inlineStr">
         <is>
           <t>API + HTML</t>
         </is>
       </c>
-      <c r="E10" s="20" t="inlineStr">
+      <c r="E11" s="21" t="inlineStr">
         <is>
           <t>https://www.junction.co.uk/wp-json/wp/v2/cj_events</t>
         </is>
       </c>
-      <c r="F10" s="20" t="inlineStr">
+      <c r="F11" s="21" t="inlineStr">
         <is>
           <t>https://www.junction.co.uk — 200; alternate-фиды: https://www.junction.co.uk/feed/, https://www.junction.co.uk/comments/feed/, https://www.junction.co.uk/wp-json/oembed/1.0/embed?url=https%3A%2F%2Fwww.junction.co.uk%2F; WordPress; билетная система: ecal, spektrix
 https://www.junction.co.uk/whats-on/ — 200; alternate-фиды: https://www.junction.co.uk/feed/, https://www.junction.co.uk/comments/feed/, https://www.junction.co.uk/wp-json/oembed/1.0/embed?url=https%3A%2F%2Fwww.junction.co.uk%2Fwhats-on%2F; WordPress; билетная система: ecal, spektrix
@@ -6659,35 +6875,35 @@
 https://www.junction.co.uk/feed/ — 200; фид, записей: 12</t>
         </is>
       </c>
-      <c r="G10" s="20" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="20" t="inlineStr">
+      <c r="G11" s="21" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="21" t="inlineStr">
         <is>
           <t>S018</t>
         </is>
       </c>
-      <c r="B11" s="20" t="inlineStr">
+      <c r="B12" s="21" t="inlineStr">
         <is>
           <t>Cambridge United</t>
         </is>
       </c>
-      <c r="C11" s="21" t="inlineStr">
+      <c r="C12" s="22" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D11" s="20" t="inlineStr">
+      <c r="D12" s="21" t="inlineStr">
         <is>
           <t>iCal (fixtur.es) + HTML</t>
         </is>
       </c>
-      <c r="E11" s="20" t="inlineStr">
+      <c r="E12" s="21" t="inlineStr">
         <is>
           <t>https://ics.fixtur.es/v2/home/cambridge-united-fc.ics</t>
         </is>
       </c>
-      <c r="F11" s="20" t="inlineStr">
+      <c r="F12" s="21" t="inlineStr">
         <is>
           <t>https://www.cambridgeunited.com — 200
 https://fixtur.es/en/team/cambridge-united-fc/home — 200; JSON-LD Event: 27
@@ -6695,372 +6911,372 @@
 https://ics.fixtur.es/v2/home/cambridge-united-fc.ics — 200; iCal, событий: 188</t>
         </is>
       </c>
-      <c r="G11" s="20" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="20" t="inlineStr">
+      <c r="G12" s="21" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="21" t="inlineStr">
         <is>
           <t>S021</t>
         </is>
       </c>
-      <c r="B12" s="20" t="inlineStr">
+      <c r="B13" s="21" t="inlineStr">
         <is>
           <t>Newmarket Racecourses</t>
         </is>
       </c>
-      <c r="C12" s="21" t="inlineStr">
+      <c r="C13" s="22" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D12" s="20" t="inlineStr">
+      <c r="D13" s="21" t="inlineStr">
         <is>
           <t>JSON-LD</t>
         </is>
       </c>
-      <c r="E12" s="20" t="inlineStr">
+      <c r="E13" s="21" t="inlineStr">
         <is>
           <t>https://www.thejockeyclub.co.uk/newmarket/events-tickets/</t>
         </is>
       </c>
-      <c r="F12" s="20" t="inlineStr">
+      <c r="F13" s="21" t="inlineStr">
         <is>
           <t>https://www.thejockeyclub.co.uk/newmarket/ — 200
 https://www.thejockeyclub.co.uk/newmarket/events-tickets/ — 200; JSON-LD Event: 14</t>
         </is>
       </c>
-      <c r="G12" s="20" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="20" t="inlineStr">
+      <c r="G13" s="21" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="21" t="inlineStr">
         <is>
           <t>S026</t>
         </is>
       </c>
-      <c r="B13" s="20" t="inlineStr">
+      <c r="B14" s="21" t="inlineStr">
         <is>
           <t>Chariots of Fire</t>
         </is>
       </c>
-      <c r="C13" s="21" t="inlineStr">
+      <c r="C14" s="22" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D13" s="20" t="inlineStr">
+      <c r="D14" s="21" t="inlineStr">
         <is>
           <t>JSON-LD (RunThrough)</t>
         </is>
       </c>
-      <c r="E13" s="20" t="inlineStr">
+      <c r="E14" s="21" t="inlineStr">
         <is>
           <t>https://www.runthrough.co.uk/event/chariots-of-fire-september-2026</t>
         </is>
       </c>
-      <c r="F13" s="20" t="inlineStr">
+      <c r="F14" s="21" t="inlineStr">
         <is>
           <t>https://www.chariots-of-fire.co.uk/ — 200; alternate-фиды: https://www.chariots-of-fire.co.uk/feed/, https://www.chariots-of-fire.co.uk/comments/feed/, https://www.chariots-of-fire.co.uk/wp-json/wp/v2/pages/21; WordPress
 https://www.chariots-of-fire.co.uk/feed/ — 200; фид, записей: 10
 https://www.runthrough.co.uk/event/chariots-of-fire-september-2026 — 200; JSON-LD Event: 1</t>
         </is>
       </c>
-      <c r="G13" s="20" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="20" t="inlineStr">
+      <c r="G14" s="21" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="21" t="inlineStr">
         <is>
           <t>S028</t>
         </is>
       </c>
-      <c r="B14" s="20" t="inlineStr">
+      <c r="B15" s="21" t="inlineStr">
         <is>
           <t>Cambridge Half Marathon</t>
         </is>
       </c>
-      <c r="C14" s="21" t="inlineStr">
+      <c r="C15" s="22" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D14" s="20" t="inlineStr">
+      <c r="D15" s="21" t="inlineStr">
         <is>
           <t>HTML</t>
         </is>
       </c>
-      <c r="E14" s="20" t="inlineStr">
+      <c r="E15" s="21" t="inlineStr">
         <is>
           <t>https://cambridgehalfmarathon.com/</t>
         </is>
       </c>
-      <c r="F14" s="20" t="inlineStr">
+      <c r="F15" s="21" t="inlineStr">
         <is>
           <t>https://cambridgehalfmarathon.com/ — 200</t>
         </is>
       </c>
-      <c r="G14" s="20" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="20" t="inlineStr">
+      <c r="G15" s="21" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="21" t="inlineStr">
         <is>
           <t>S030</t>
         </is>
       </c>
-      <c r="B15" s="20" t="inlineStr">
+      <c r="B16" s="21" t="inlineStr">
         <is>
           <t>Cambridge Festival (университет)</t>
         </is>
       </c>
-      <c r="C15" s="21" t="inlineStr">
+      <c r="C16" s="22" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D15" s="20" t="inlineStr">
+      <c r="D16" s="21" t="inlineStr">
+        <is>
+          <t>HTML (curl, пауза 10 с)</t>
+        </is>
+      </c>
+      <c r="E16" s="21" t="inlineStr">
+        <is>
+          <t>https://www.festival.cam.ac.uk/events</t>
+        </is>
+      </c>
+      <c r="F16" s="21" t="inlineStr">
+        <is>
+          <t>https://www.festival.cam.ac.uk/events — 200 через curl, robots.txt разрешает (Crawl-delay: 10); фидов и JSON-LD нет</t>
+        </is>
+      </c>
+      <c r="G16" s="21" t="inlineStr">
+        <is>
+          <t>Pantheon отдаёт 403 Python-клиенту httpx (и на robots.txt), curl с тем же User-Agent — 200: блок по отпечатку клиента</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="21" t="inlineStr">
+        <is>
+          <t>S031</t>
+        </is>
+      </c>
+      <c r="B17" s="21" t="inlineStr">
+        <is>
+          <t>Cambridge Folk Festival</t>
+        </is>
+      </c>
+      <c r="C17" s="22" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="D17" s="21" t="inlineStr">
         <is>
           <t>HTML</t>
         </is>
       </c>
-      <c r="E15" s="20" t="inlineStr">
-        <is>
-          <t>https://www.festival.cam.ac.uk/events</t>
-        </is>
-      </c>
-      <c r="F15" s="20" t="inlineStr">
-        <is>
-          <t>https://www.festival.cam.ac.uk/events — 200 через curl, robots.txt разрешает (Crawl-delay: 10); фидов и JSON-LD нет</t>
-        </is>
-      </c>
-      <c r="G15" s="20" t="inlineStr">
-        <is>
-          <t>Pantheon отдаёт 403 Python-клиенту httpx (и на robots.txt), curl с тем же User-Agent — 200: блок по отпечатку клиента</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="20" t="inlineStr">
-        <is>
-          <t>S031</t>
-        </is>
-      </c>
-      <c r="B16" s="20" t="inlineStr">
-        <is>
-          <t>Cambridge Folk Festival</t>
-        </is>
-      </c>
-      <c r="C16" s="21" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
-      <c r="D16" s="20" t="inlineStr">
-        <is>
-          <t>HTML</t>
-        </is>
-      </c>
-      <c r="E16" s="20" t="inlineStr">
+      <c r="E17" s="21" t="inlineStr">
         <is>
           <t>https://www.cambridgefolkfestival.co.uk/</t>
         </is>
       </c>
-      <c r="F16" s="20" t="inlineStr">
+      <c r="F17" s="21" t="inlineStr">
         <is>
           <t>https://www.cambridgefolkfestival.co.uk/ — 200
 https://www.cambridgefolkfestival.co.uk/ — 200</t>
         </is>
       </c>
-      <c r="G16" s="20" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="20" t="inlineStr">
+      <c r="G17" s="21" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="21" t="inlineStr">
         <is>
           <t>S032</t>
         </is>
       </c>
-      <c r="B17" s="20" t="inlineStr">
+      <c r="B18" s="21" t="inlineStr">
         <is>
           <t>Cambridge Beer Festival</t>
         </is>
       </c>
-      <c r="C17" s="21" t="inlineStr">
+      <c r="C18" s="22" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D17" s="20" t="inlineStr">
+      <c r="D18" s="21" t="inlineStr">
         <is>
           <t>iCal</t>
         </is>
       </c>
-      <c r="E17" s="20" t="inlineStr">
+      <c r="E18" s="21" t="inlineStr">
         <is>
           <t>https://www.cambridgebeerfestival.com/events/?ical=1</t>
         </is>
       </c>
-      <c r="F17" s="20" t="inlineStr">
+      <c r="F18" s="21" t="inlineStr">
         <is>
           <t>https://www.cambridgebeerfestival.com — 200; JSON-LD Event: 2; alternate-фиды: https://www.cambridgebeerfestival.com/events/?ical=1; WordPress + The Events Calendar; билетная система: ecal</t>
         </is>
       </c>
-      <c r="G17" s="20" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="20" t="inlineStr">
+      <c r="G18" s="21" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="21" t="inlineStr">
         <is>
           <t>S033</t>
         </is>
       </c>
-      <c r="B18" s="20" t="inlineStr">
+      <c r="B19" s="21" t="inlineStr">
         <is>
           <t>Strawberry Fair</t>
         </is>
       </c>
-      <c r="C18" s="21" t="inlineStr">
+      <c r="C19" s="22" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D18" s="20" t="inlineStr">
+      <c r="D19" s="21" t="inlineStr">
         <is>
           <t>JSON-LD</t>
         </is>
       </c>
-      <c r="E18" s="20" t="inlineStr">
+      <c r="E19" s="21" t="inlineStr">
         <is>
           <t>https://strawberry-fair.org.uk/</t>
         </is>
       </c>
-      <c r="F18" s="20" t="inlineStr">
+      <c r="F19" s="21" t="inlineStr">
         <is>
           <t>https://strawberry-fair.org.uk/ — 200; JSON-LD Event: 1
 https://strawberry-fair.org.uk/feed/ — 200; JSON-LD Event: 1</t>
         </is>
       </c>
-      <c r="G18" s="20" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="20" t="inlineStr">
+      <c r="G19" s="21" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="21" t="inlineStr">
         <is>
           <t>S038</t>
         </is>
       </c>
-      <c r="B19" s="20" t="inlineStr">
+      <c r="B20" s="21" t="inlineStr">
         <is>
           <t>Mill Road Winter Fair</t>
         </is>
       </c>
-      <c r="C19" s="21" t="inlineStr">
+      <c r="C20" s="22" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D19" s="20" t="inlineStr">
+      <c r="D20" s="21" t="inlineStr">
         <is>
           <t>RSS</t>
         </is>
       </c>
-      <c r="E19" s="20" t="inlineStr">
+      <c r="E20" s="21" t="inlineStr">
         <is>
           <t>https://www.millroadwinterfair.org/feed/</t>
         </is>
       </c>
-      <c r="F19" s="20" t="inlineStr">
+      <c r="F20" s="21" t="inlineStr">
         <is>
           <t>https://www.millroadwinterfair.org — 200; alternate-фиды: https://www.millroadwinterfair.org/feed/, https://www.millroadwinterfair.org/comments/feed/, https://www.millroadwinterfair.org/wp-json/wp/v2/pages/22; WordPress
 https://www.millroadwinterfair.org/feed/ — 200; фид, записей: 0</t>
         </is>
       </c>
-      <c r="G19" s="20" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="20" t="inlineStr">
+      <c r="G20" s="21" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="21" t="inlineStr">
         <is>
           <t>S039</t>
         </is>
       </c>
-      <c r="B20" s="20" t="inlineStr">
+      <c r="B21" s="21" t="inlineStr">
         <is>
           <t>Рождественские маркеты в центре</t>
         </is>
       </c>
-      <c r="C20" s="21" t="inlineStr">
+      <c r="C21" s="22" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D20" s="20" t="inlineStr">
+      <c r="D21" s="21" t="inlineStr">
         <is>
           <t>HTML</t>
         </is>
       </c>
-      <c r="E20" s="20" t="inlineStr">
+      <c r="E21" s="21" t="inlineStr">
         <is>
           <t>https://www.christmasincambridge.co.uk/</t>
         </is>
       </c>
-      <c r="F20" s="20" t="inlineStr">
+      <c r="F21" s="21" t="inlineStr">
         <is>
           <t>https://www.christmasincambridge.co.uk/ — 200
 https://www.visitcambridge.org/event/christmas-in-cambridge/ — 200; alternate-фиды: https://www.visitcambridge.org/wp-json/oembed/1.0/embed?url=https%3A%2F%2Fwww.visitcambridge.org%2Fevent%2Fchristmas-in-cambridge%2F; WordPress</t>
         </is>
       </c>
-      <c r="G20" s="20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="20" t="inlineStr">
+      <c r="G21" s="21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="21" t="inlineStr">
         <is>
           <t>S041</t>
         </is>
       </c>
-      <c r="B21" s="20" t="inlineStr">
+      <c r="B22" s="21" t="inlineStr">
         <is>
           <t>Cambridge Arts Theatre</t>
         </is>
       </c>
-      <c r="C21" s="22" t="inlineStr">
+      <c r="C22" s="23" t="inlineStr">
         <is>
           <t>проверить</t>
         </is>
       </c>
-      <c r="D21" s="20" t="inlineStr">
-        <is>
-          <t>HTML (блок Cloudflare)</t>
-        </is>
-      </c>
-      <c r="E21" s="20" t="inlineStr"/>
-      <c r="F21" s="20" t="inlineStr"/>
-      <c r="G21" s="20" t="inlineStr">
+      <c r="D22" s="21" t="inlineStr">
+        <is>
+          <t>Через Ents24 (S006)</t>
+        </is>
+      </c>
+      <c r="E22" s="21" t="inlineStr"/>
+      <c r="F22" s="21" t="inlineStr"/>
+      <c r="G22" s="21" t="inlineStr">
         <is>
           <t>https://www.artstheatre.co.uk — 403, Cloudflare challenge (cf-mitigated) и для httpx, и для curl</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="20" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="21" t="inlineStr">
         <is>
           <t>S042</t>
         </is>
       </c>
-      <c r="B22" s="20" t="inlineStr">
+      <c r="B23" s="21" t="inlineStr">
         <is>
           <t>ADC Theatre</t>
         </is>
       </c>
-      <c r="C22" s="21" t="inlineStr">
+      <c r="C23" s="22" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D22" s="20" t="inlineStr">
+      <c r="D23" s="21" t="inlineStr">
         <is>
           <t>iCal</t>
         </is>
       </c>
-      <c r="E22" s="20" t="inlineStr">
+      <c r="E23" s="21" t="inlineStr">
         <is>
           <t>https://www.camdram.net/venues/adc-theatre/diary.ics</t>
         </is>
       </c>
-      <c r="F22" s="20" t="inlineStr">
+      <c r="F23" s="21" t="inlineStr">
         <is>
           <t>https://www.adctheatre.com — 200; билетная система: spektrix
 https://www.adctheatre.com/whats-on/ — 200; билетная система: spektrix
@@ -7068,184 +7284,186 @@
 https://www.camdram.net/venues/adc-theatre/diary.json — 200; JSON</t>
         </is>
       </c>
-      <c r="G22" s="20" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="20" t="inlineStr">
+      <c r="G23" s="21" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="21" t="inlineStr">
         <is>
           <t>S045</t>
         </is>
       </c>
-      <c r="B23" s="20" t="inlineStr">
+      <c r="B24" s="21" t="inlineStr">
         <is>
           <t>Arts Picturehouse</t>
         </is>
       </c>
-      <c r="C23" s="21" t="inlineStr">
+      <c r="C24" s="22" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D23" s="20" t="inlineStr">
+      <c r="D24" s="21" t="inlineStr">
         <is>
           <t>HTML</t>
         </is>
       </c>
-      <c r="E23" s="20" t="inlineStr">
+      <c r="E24" s="21" t="inlineStr">
         <is>
           <t>https://www.picturehouses.com/cinema/arts-picturehouse-cambridge</t>
         </is>
       </c>
-      <c r="F23" s="20" t="inlineStr">
+      <c r="F24" s="21" t="inlineStr">
         <is>
           <t>https://www.picturehouses.com/cinema/arts-picturehouse-cambridge — 200; билетная система: ecal</t>
         </is>
       </c>
-      <c r="G23" s="20" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="20" t="inlineStr">
+      <c r="G24" s="21" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="21" t="inlineStr">
         <is>
           <t>S047</t>
         </is>
       </c>
-      <c r="B24" s="20" t="inlineStr">
+      <c r="B25" s="21" t="inlineStr">
         <is>
           <t>Talks.cam</t>
         </is>
       </c>
-      <c r="C24" s="21" t="inlineStr">
+      <c r="C25" s="22" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D24" s="20" t="inlineStr">
+      <c r="D25" s="21" t="inlineStr">
         <is>
           <t>iCal</t>
         </is>
       </c>
-      <c r="E24" s="20" t="inlineStr">
-        <is>
-          <t>https://talks.cam.ac.uk/show/ics/5606/</t>
-        </is>
-      </c>
-      <c r="F24" s="20" t="inlineStr">
+      <c r="E25" s="21" t="inlineStr">
+        <is>
+          <t>https://talks.cam.ac.uk/show/ics/{5606,5462,5358,5769,23088}/</t>
+        </is>
+      </c>
+      <c r="F25" s="21" t="inlineStr">
         <is>
           <t>https://talks.cam.ac.uk — 200
 https://talks.cam.ac.uk/document/documentation/ — 200
 https://talks.cam.ac.uk/show/ics/5606/ — 200; iCal, событий: 15
-https://talks.cam.ac.uk/show/rss/5606/ — 200; фид, записей: 15
-https://talks.cam.ac.uk/show/xml/5606/ — 200</t>
-        </is>
-      </c>
-      <c r="G24" s="20" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="20" t="inlineStr">
+https://talks.cam.ac.uk/show/ics/5462/ — 200; iCal, событий: 8
+https://talks.cam.ac.uk/show/ics/5358/ — 200; iCal, событий: 8
+https://talks.cam.ac.uk/show/ics/5769/ — 200; iCal, событий: 7
+https://talks.cam.ac.uk/show/ics/23088/ — 200; iCal, событий: 55</t>
+        </is>
+      </c>
+      <c r="G25" s="21" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="21" t="inlineStr">
         <is>
           <t>S048</t>
         </is>
       </c>
-      <c r="B25" s="20" t="inlineStr">
+      <c r="B26" s="21" t="inlineStr">
         <is>
           <t>University of Cambridge — What's On</t>
         </is>
       </c>
-      <c r="C25" s="21" t="inlineStr">
+      <c r="C26" s="22" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D25" s="20" t="inlineStr">
+      <c r="D26" s="21" t="inlineStr">
         <is>
           <t>HTML</t>
         </is>
       </c>
-      <c r="E25" s="20" t="inlineStr">
+      <c r="E26" s="21" t="inlineStr">
         <is>
           <t>https://www.admin.cam.ac.uk/whatson/</t>
         </is>
       </c>
-      <c r="F25" s="20" t="inlineStr">
+      <c r="F26" s="21" t="inlineStr">
         <is>
           <t>https://www.admin.cam.ac.uk/whatson/ — 200</t>
         </is>
       </c>
-      <c r="G25" s="20" t="inlineStr">
+      <c r="G26" s="21" t="inlineStr">
         <is>
           <t>webservices.admin.cam.ac.uk (iCal 76 событий, RSS) — robots.txt: Disallow: / — не собираем без решения
 https://www.cam.ac.uk/whats-on — Pantheon 403 для httpx</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="20" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="21" t="inlineStr">
         <is>
           <t>S050</t>
         </is>
       </c>
-      <c r="B26" s="20" t="inlineStr">
+      <c r="B27" s="21" t="inlineStr">
         <is>
           <t>Fitzwilliam Museum</t>
         </is>
       </c>
-      <c r="C26" s="21" t="inlineStr">
+      <c r="C27" s="22" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D26" s="20" t="inlineStr">
+      <c r="D27" s="21" t="inlineStr">
         <is>
           <t>RSS (выставки) + HTML (события)</t>
         </is>
       </c>
-      <c r="E26" s="20" t="inlineStr">
+      <c r="E27" s="21" t="inlineStr">
         <is>
           <t>https://fitzmuseum.cam.ac.uk/feeds/exhibitions</t>
         </is>
       </c>
-      <c r="F26" s="20" t="inlineStr">
+      <c r="F27" s="21" t="inlineStr">
         <is>
           <t>https://fitzmuseum.cam.ac.uk — 200; alternate-фиды: https://fitzmuseum.cam.ac.uk/feeds/news, https://fitzmuseum.cam.ac.uk/feeds/vacancies, https://fitzmuseum.cam.ac.uk/feeds/exhibitions
 https://fitzmuseum.cam.ac.uk/events — 200; alternate-фиды: https://fitzmuseum.cam.ac.uk/feeds/news, https://fitzmuseum.cam.ac.uk/feeds/vacancies, https://fitzmuseum.cam.ac.uk/feeds/exhibitions
 https://fitzmuseum.cam.ac.uk/feeds/exhibitions — 200; фид, записей: 20</t>
         </is>
       </c>
-      <c r="G26" s="20" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="20" t="inlineStr">
+      <c r="G27" s="21" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="21" t="inlineStr">
         <is>
           <t>S051</t>
         </is>
       </c>
-      <c r="B27" s="20" t="inlineStr">
+      <c r="B28" s="21" t="inlineStr">
         <is>
           <t>Kettle's Yard</t>
         </is>
       </c>
-      <c r="C27" s="21" t="inlineStr">
+      <c r="C28" s="22" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D27" s="20" t="inlineStr">
+      <c r="D28" s="21" t="inlineStr">
         <is>
           <t>HTML</t>
         </is>
       </c>
-      <c r="E27" s="20" t="inlineStr">
+      <c r="E28" s="21" t="inlineStr">
         <is>
           <t>https://www.kettlesyard.cam.ac.uk/whats-on/</t>
         </is>
       </c>
-      <c r="F27" s="20" t="inlineStr">
+      <c r="F28" s="21" t="inlineStr">
         <is>
           <t>https://www.kettlesyard.cam.ac.uk — 200
 https://www.kettlesyard.cam.ac.uk/whats-on/ — 200</t>
         </is>
       </c>
-      <c r="G27" s="20" t="inlineStr">
+      <c r="G28" s="21" t="inlineStr">
         <is>
           <t>https://www.kettlesyard.cam.ac.uk/feed/ — 500
 https://www.kettlesyard.co.uk — ConnectError: [SSL: CERTIFICATE_VERIFY_FAILED] certificate verify failed: Hostname mismatch, certificate is not valid for 'www.kettlesyard.co.uk'. (_ssl.c:1016)
@@ -7254,389 +7472,726 @@
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="20" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="21" t="inlineStr">
         <is>
           <t>S052</t>
         </is>
       </c>
-      <c r="B28" s="20" t="inlineStr">
+      <c r="B29" s="21" t="inlineStr">
         <is>
           <t>University of Cambridge Museums (сводный)</t>
         </is>
       </c>
-      <c r="C28" s="21" t="inlineStr">
+      <c r="C29" s="22" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D28" s="20" t="inlineStr">
+      <c r="D29" s="21" t="inlineStr">
         <is>
           <t>HTML</t>
         </is>
       </c>
-      <c r="E28" s="20" t="inlineStr">
+      <c r="E29" s="21" t="inlineStr">
         <is>
           <t>https://www.museums.cam.ac.uk/whats-on</t>
         </is>
       </c>
-      <c r="F28" s="20" t="inlineStr">
+      <c r="F29" s="21" t="inlineStr">
         <is>
           <t>https://www.museums.cam.ac.uk — 200
 https://www.museums.cam.ac.uk/whats-on — 200</t>
         </is>
       </c>
-      <c r="G28" s="20" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="20" t="inlineStr">
+      <c r="G29" s="21" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="21" t="inlineStr">
         <is>
           <t>S056</t>
         </is>
       </c>
-      <c r="B29" s="20" t="inlineStr">
+      <c r="B30" s="21" t="inlineStr">
         <is>
           <t>Семейные программы музеев</t>
         </is>
       </c>
-      <c r="C29" s="22" t="inlineStr">
+      <c r="C30" s="23" t="inlineStr">
         <is>
           <t>проверить</t>
         </is>
       </c>
-      <c r="D29" s="20" t="inlineStr">
+      <c r="D30" s="21" t="inlineStr">
         <is>
           <t>Производный (тег «дети»)</t>
         </is>
       </c>
-      <c r="E29" s="20" t="inlineStr"/>
-      <c r="F29" s="20" t="inlineStr"/>
-      <c r="G29" s="20" t="inlineStr">
+      <c r="E30" s="21" t="inlineStr"/>
+      <c r="F30" s="21" t="inlineStr"/>
+      <c r="G30" s="21" t="inlineStr">
         <is>
           <t>своего URL нет по замыслу</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="20" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="21" t="inlineStr">
         <is>
           <t>S062</t>
         </is>
       </c>
-      <c r="B30" s="20" t="inlineStr">
+      <c r="B31" s="21" t="inlineStr">
         <is>
           <t>Комедия на Corn Exchange / Junction / ADC</t>
         </is>
       </c>
-      <c r="C30" s="22" t="inlineStr">
+      <c r="C31" s="23" t="inlineStr">
         <is>
           <t>проверить</t>
         </is>
       </c>
-      <c r="D30" s="20" t="inlineStr">
+      <c r="D31" s="21" t="inlineStr">
         <is>
           <t>Производный (тег «комедия»)</t>
         </is>
       </c>
-      <c r="E30" s="20" t="inlineStr"/>
-      <c r="F30" s="20" t="inlineStr"/>
-      <c r="G30" s="20" t="inlineStr">
+      <c r="E31" s="21" t="inlineStr"/>
+      <c r="F31" s="21" t="inlineStr"/>
+      <c r="G31" s="21" t="inlineStr">
         <is>
           <t>своего URL нет по замыслу</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="20" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="21" t="inlineStr">
         <is>
           <t>S065</t>
         </is>
       </c>
-      <c r="B31" s="20" t="inlineStr">
+      <c r="B32" s="21" t="inlineStr">
         <is>
           <t>Open Cambridge</t>
         </is>
       </c>
-      <c r="C31" s="21" t="inlineStr">
+      <c r="C32" s="22" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D31" s="20" t="inlineStr">
+      <c r="D32" s="21" t="inlineStr">
+        <is>
+          <t>HTML (curl, пауза 10 с)</t>
+        </is>
+      </c>
+      <c r="E32" s="21" t="inlineStr">
+        <is>
+          <t>https://www.opencambridge.cam.ac.uk/</t>
+        </is>
+      </c>
+      <c r="F32" s="21" t="inlineStr">
+        <is>
+          <t>https://www.opencambridge.cam.ac.uk/ — 200 через curl; фидов нет</t>
+        </is>
+      </c>
+      <c r="G32" s="21" t="inlineStr">
+        <is>
+          <t>Pantheon отдаёт 403 Python-клиенту httpx, curl — 200</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="21" t="inlineStr">
+        <is>
+          <t>S069</t>
+        </is>
+      </c>
+      <c r="B33" s="21" t="inlineStr">
+        <is>
+          <t>Cambridge University Botanic Garden</t>
+        </is>
+      </c>
+      <c r="C33" s="22" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="D33" s="21" t="inlineStr">
         <is>
           <t>HTML</t>
         </is>
       </c>
-      <c r="E31" s="20" t="inlineStr">
-        <is>
-          <t>https://www.opencambridge.cam.ac.uk/</t>
-        </is>
-      </c>
-      <c r="F31" s="20" t="inlineStr">
-        <is>
-          <t>https://www.opencambridge.cam.ac.uk/ — 200 через curl; фидов нет</t>
-        </is>
-      </c>
-      <c r="G31" s="20" t="inlineStr">
-        <is>
-          <t>Pantheon отдаёт 403 Python-клиенту httpx, curl — 200</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="20" t="inlineStr">
-        <is>
-          <t>S069</t>
-        </is>
-      </c>
-      <c r="B32" s="20" t="inlineStr">
-        <is>
-          <t>Cambridge University Botanic Garden</t>
-        </is>
-      </c>
-      <c r="C32" s="21" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
-      <c r="D32" s="20" t="inlineStr">
-        <is>
-          <t>HTML</t>
-        </is>
-      </c>
-      <c r="E32" s="20" t="inlineStr">
+      <c r="E33" s="21" t="inlineStr">
         <is>
           <t>https://www.botanic.cam.ac.uk/whats-on/</t>
         </is>
       </c>
-      <c r="F32" s="20" t="inlineStr">
+      <c r="F33" s="21" t="inlineStr">
         <is>
           <t>https://www.botanic.cam.ac.uk — 200; alternate-фиды: https://www.botanic.cam.ac.uk/wp-json/oembed/1.0/embed?url=https%3A%2F%2Fwww.botanic.cam.ac.uk%2F, https://www.botanic.cam.ac.uk/wp-json/wp/v2/pages/6; WordPress
 https://www.botanic.cam.ac.uk/whats-on/ — 200; WordPress</t>
         </is>
       </c>
-      <c r="G32" s="20" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="20" t="inlineStr">
+      <c r="G33" s="21" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="21" t="inlineStr">
         <is>
           <t>S070</t>
         </is>
       </c>
-      <c r="B33" s="20" t="inlineStr">
+      <c r="B34" s="21" t="inlineStr">
         <is>
           <t>National Trust: Wimpole, Anglesey Abbey, Wicken Fen</t>
         </is>
       </c>
-      <c r="C33" s="22" t="inlineStr">
+      <c r="C34" s="23" t="inlineStr">
         <is>
           <t>проверить</t>
         </is>
       </c>
-      <c r="D33" s="20" t="inlineStr">
-        <is>
-          <t>HTML</t>
-        </is>
-      </c>
-      <c r="E33" s="20" t="inlineStr">
+      <c r="D34" s="21" t="inlineStr">
+        <is>
+          <t>Ручной сезонный</t>
+        </is>
+      </c>
+      <c r="E34" s="21" t="inlineStr">
         <is>
           <t>https://www.nationaltrust.org.uk/visit/cambridgeshire/wimpole-estate/events</t>
         </is>
       </c>
-      <c r="F33" s="20" t="inlineStr">
+      <c r="F34" s="21" t="inlineStr">
         <is>
           <t>https://www.nationaltrust.org.uk/visit/cambridgeshire/wimpole-estate/events — 200
 https://www.nationaltrust.org.uk/visit/cambridgeshire/anglesey-abbey-gardens-and-lode-mill/events — 200
 https://www.nationaltrust.org.uk/visit/cambridgeshire/wicken-fen-nature-reserve/events — 200</t>
         </is>
       </c>
-      <c r="G33" s="20" t="inlineStr">
+      <c r="G34" s="21" t="inlineStr">
         <is>
           <t>nationaltrust.org.uk — после 1–2 запросов отдаёт страницу бот-защиты Radware
 Wicken Fen: /wicken-fen-nature-reserve/events — страница 404; верный адрес не подтверждён</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="20" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="21" t="inlineStr">
         <is>
           <t>S072</t>
         </is>
       </c>
-      <c r="B34" s="20" t="inlineStr">
+      <c r="B35" s="21" t="inlineStr">
         <is>
           <t>Cambridge City Council — городские события</t>
         </is>
       </c>
-      <c r="C34" s="21" t="inlineStr">
+      <c r="C35" s="22" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D34" s="20" t="inlineStr">
+      <c r="D35" s="21" t="inlineStr">
         <is>
           <t>HTML</t>
         </is>
       </c>
-      <c r="E34" s="20" t="inlineStr">
+      <c r="E35" s="21" t="inlineStr">
         <is>
           <t>https://www.camcityevents.co.uk/events</t>
         </is>
       </c>
-      <c r="F34" s="20" t="inlineStr">
+      <c r="F35" s="21" t="inlineStr">
         <is>
           <t>https://www.cambridge.gov.uk — 200
 https://www.cambridge.gov.uk/summer-events — 200
 https://www.camcityevents.co.uk/events — 200</t>
         </is>
       </c>
-      <c r="G34" s="20" t="inlineStr">
+      <c r="G35" s="21" t="inlineStr">
         <is>
           <t>https://www.cambridge.gov.uk/fireworks — 404</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="20" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="21" t="inlineStr">
         <is>
           <t>S081</t>
         </is>
       </c>
-      <c r="B35" s="20" t="inlineStr">
+      <c r="B36" s="21" t="inlineStr">
         <is>
           <t>Thriplow Daffodil Weekend</t>
         </is>
       </c>
-      <c r="C35" s="21" t="inlineStr">
+      <c r="C36" s="22" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D35" s="20" t="inlineStr">
+      <c r="D36" s="21" t="inlineStr">
         <is>
           <t>HTML</t>
         </is>
       </c>
-      <c r="E35" s="20" t="inlineStr">
+      <c r="E36" s="21" t="inlineStr">
         <is>
           <t>https://www.thriplowdaffodils.org.uk</t>
         </is>
       </c>
-      <c r="F35" s="20" t="inlineStr">
+      <c r="F36" s="21" t="inlineStr">
         <is>
           <t>https://www.thriplowdaffodils.org.uk — 200</t>
         </is>
       </c>
-      <c r="G35" s="20" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="20" t="inlineStr">
+      <c r="G36" s="21" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="21" t="inlineStr">
         <is>
           <t>S082</t>
         </is>
       </c>
-      <c r="B36" s="20" t="inlineStr">
+      <c r="B37" s="21" t="inlineStr">
         <is>
           <t>Cambridge Dragon Boat Festival (ACT)</t>
         </is>
       </c>
-      <c r="C36" s="21" t="inlineStr">
+      <c r="C37" s="22" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D36" s="20" t="inlineStr">
+      <c r="D37" s="21" t="inlineStr">
         <is>
           <t>HTML</t>
         </is>
       </c>
-      <c r="E36" s="20" t="inlineStr">
+      <c r="E37" s="21" t="inlineStr">
         <is>
           <t>https://act4addenbrookes.org.uk/dragonboat/</t>
         </is>
       </c>
-      <c r="F36" s="20" t="inlineStr">
+      <c r="F37" s="21" t="inlineStr">
         <is>
           <t>https://act4addenbrookes.org.uk — 200; alternate-фиды: https://act4addenbrookes.org.uk/feed/, https://act4addenbrookes.org.uk/comments/feed/, https://act4addenbrookes.org.uk/wp-json/oembed/1.0/embed?url=https%3A%2F%2Fact4addenbrookes.org.uk%2F; WordPress
 https://act4addenbrookes.org.uk/events/cambridge-dragon-boat-festival-2026/ — 200; alternate-фиды: https://act4addenbrookes.org.uk/feed/, https://act4addenbrookes.org.uk/comments/feed/, https://act4addenbrookes.org.uk/wp-json/oembed/1.0/embed?url=https%3A%2F%2Fact4addenbrookes.org.uk%2Fevents%2Fcambridge-dragon-boat-festival-2026%2F; WordPress</t>
         </is>
       </c>
-      <c r="G36" s="20" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="20" t="inlineStr">
+      <c r="G37" s="21" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="21" t="inlineStr">
         <is>
           <t>S087</t>
         </is>
       </c>
-      <c r="B37" s="20" t="inlineStr">
+      <c r="B38" s="21" t="inlineStr">
         <is>
           <t>The Cambridge Foodies</t>
         </is>
       </c>
-      <c r="C37" s="21" t="inlineStr">
+      <c r="C38" s="22" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D37" s="20" t="inlineStr">
+      <c r="D38" s="21" t="inlineStr">
         <is>
           <t>RSS</t>
         </is>
       </c>
-      <c r="E37" s="20" t="inlineStr">
+      <c r="E38" s="21" t="inlineStr">
         <is>
           <t>https://cambridgefoodies.me.uk/feed/</t>
         </is>
       </c>
-      <c r="F37" s="20" t="inlineStr">
+      <c r="F38" s="21" t="inlineStr">
         <is>
           <t>https://cambridgefoodies.me.uk — 200 в первом проходе, WordPress, alternate RSS /feed/
 https://cambridgefoodies.me.uk/feed/ — 200 через HTTP/2</t>
         </is>
       </c>
-      <c r="G37" s="20" t="inlineStr">
+      <c r="G38" s="21" t="inlineStr">
         <is>
           <t>WordPress.com отвечает 429 при повторных запросах (и HTTP/1.1-клиенту httpx) — нужны HTTP/2, редкие запросы и бэк-офф</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="20" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="21" t="inlineStr">
         <is>
           <t>S089</t>
         </is>
       </c>
-      <c r="B38" s="20" t="inlineStr">
+      <c r="B39" s="21" t="inlineStr">
         <is>
           <t>Town and Gown 10k</t>
         </is>
       </c>
-      <c r="C38" s="22" t="inlineStr">
+      <c r="C39" s="23" t="inlineStr">
         <is>
           <t>проверить</t>
         </is>
       </c>
-      <c r="D38" s="20" t="inlineStr">
-        <is>
-          <t>Ручной (сайт закрыт для ботов)</t>
-        </is>
-      </c>
-      <c r="E38" s="20" t="inlineStr"/>
-      <c r="F38" s="20" t="inlineStr"/>
-      <c r="G38" s="20" t="inlineStr">
+      <c r="D39" s="21" t="inlineStr">
+        <is>
+          <t>Через Cambridge News (S004) и Cambridge 105 (S005)</t>
+        </is>
+      </c>
+      <c r="E39" s="21" t="inlineStr"/>
+      <c r="F39" s="21" t="inlineStr"/>
+      <c r="G39" s="21" t="inlineStr">
         <is>
           <t>townandgown10k.com и musculardystrophyuk.org — Cloudflare 403 для любого бот-клиента, включая robots.txt</t>
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" s="21" t="inlineStr">
+        <is>
+          <t>S090</t>
+        </is>
+      </c>
+      <c r="B40" s="21" t="inlineStr">
+        <is>
+          <t>DesignMyNight — Cambridge</t>
+        </is>
+      </c>
+      <c r="C40" s="24" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="D40" s="21" t="inlineStr">
+        <is>
+          <t>— (robots.txt запрещает)</t>
+        </is>
+      </c>
+      <c r="E40" s="21" t="inlineStr">
+        <is>
+          <t>https://www.designmynight.com/cambridge</t>
+        </is>
+      </c>
+      <c r="F40" s="21" t="inlineStr">
+        <is>
+          <t>https://www.designmynight.com/cambridge — 200</t>
+        </is>
+      </c>
+      <c r="G40" s="21" t="inlineStr">
+        <is>
+          <t>robots.txt: Disallow: /cambridge/whats-on и Disallow: /api/ — раздел событий закрыт для роботов
+разрешённые страницы /cambridge — каталог заведений, событий и JSON-LD Event нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="21" t="inlineStr">
+        <is>
+          <t>S091</t>
+        </is>
+      </c>
+      <c r="B41" s="21" t="inlineStr">
+        <is>
+          <t>Cambridge Live Tickets</t>
+        </is>
+      </c>
+      <c r="C41" s="22" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="D41" s="21" t="inlineStr">
+        <is>
+          <t>HTML + JSON-LD</t>
+        </is>
+      </c>
+      <c r="E41" s="21" t="inlineStr">
+        <is>
+          <t>https://www.cambridgelivetickets.co.uk/events</t>
+        </is>
+      </c>
+      <c r="F41" s="21" t="inlineStr">
+        <is>
+          <t>https://www.cambridgelivetickets.co.uk — 200
+https://www.cambridgelivetickets.co.uk/events — 200
+https://www.cambridgelivetickets.co.uk/events/georgie-carroll-nurse-georgie-carroll-infectious — 200; JSON-LD Event: 1</t>
+        </is>
+      </c>
+      <c r="G41" s="21" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G38"/>
+  <autoFilter ref="A1:G41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" style="11" min="1" max="1"/>
+    <col width="44" customWidth="1" style="11" min="2" max="2"/>
+    <col width="22" customWidth="1" style="11" min="3" max="3"/>
+    <col width="60" customWidth="1" style="11" min="4" max="4"/>
+    <col width="36" customWidth="1" style="11" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="20" t="inlineStr">
+        <is>
+          <t>Событие</t>
+        </is>
+      </c>
+      <c r="C1" s="20" t="inlineStr">
+        <is>
+          <t>Когда</t>
+        </is>
+      </c>
+      <c r="D1" s="20" t="inlineStr">
+        <is>
+          <t>Где искать</t>
+        </is>
+      </c>
+      <c r="E1" s="20" t="inlineStr">
+        <is>
+          <t>Ключевые слова</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="21" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="B2" s="21" t="inlineStr">
+        <is>
+          <t>Домашние матчи Cambridge United</t>
+        </is>
+      </c>
+      <c r="C2" s="21" t="inlineStr">
+        <is>
+          <t>весь сезон</t>
+        </is>
+      </c>
+      <c r="D2" s="21" t="inlineStr">
+        <is>
+          <t>S018 (fixtur.es), будущие домашние матчи</t>
+        </is>
+      </c>
+      <c r="E2" s="21" t="inlineStr">
+        <is>
+          <t>Cambridge United</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="21" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="B3" s="21" t="inlineStr">
+        <is>
+          <t>Mill Road Winter Fair</t>
+        </is>
+      </c>
+      <c r="C3" s="21" t="inlineStr">
+        <is>
+          <t>2026-12-05</t>
+        </is>
+      </c>
+      <c r="D3" s="21" t="inlineStr">
+        <is>
+          <t>S038 (сайт ярмарки), Cambridge 105, Cambridge News</t>
+        </is>
+      </c>
+      <c r="E3" s="21" t="inlineStr">
+        <is>
+          <t>Mill Road Winter Fair</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="21" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="inlineStr">
+        <is>
+          <t>Town and Gown 10k</t>
+        </is>
+      </c>
+      <c r="C4" s="21" t="inlineStr">
+        <is>
+          <t>октябрь 2026</t>
+        </is>
+      </c>
+      <c r="D4" s="21" t="inlineStr">
+        <is>
+          <t>через Cambridge News (S004) и Cambridge 105 (S005) — сайт закрыт для ботов</t>
+        </is>
+      </c>
+      <c r="E4" s="21" t="inlineStr">
+        <is>
+          <t>Town and Gown, Town &amp; Gown, Bidwells Cambridge 10k</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="21" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="B5" s="21" t="inlineStr">
+        <is>
+          <t>Whittlesea Straw Bear Festival</t>
+        </is>
+      </c>
+      <c r="C5" s="21" t="inlineStr">
+        <is>
+          <t>январь 2027</t>
+        </is>
+      </c>
+      <c r="D5" s="21" t="inlineStr">
+        <is>
+          <t>Cambridge 105, Visit Cambridge, новости</t>
+        </is>
+      </c>
+      <c r="E5" s="21" t="inlineStr">
+        <is>
+          <t>Straw Bear</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="21" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="B6" s="21" t="inlineStr">
+        <is>
+          <t>Thriplow Daffodil Weekend</t>
+        </is>
+      </c>
+      <c r="C6" s="21" t="inlineStr">
+        <is>
+          <t>март 2027</t>
+        </is>
+      </c>
+      <c r="D6" s="21" t="inlineStr">
+        <is>
+          <t>Cambridge 105</t>
+        </is>
+      </c>
+      <c r="E6" s="21" t="inlineStr">
+        <is>
+          <t>Thriplow, Daffodil Weekend</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="21" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="B7" s="21" t="inlineStr">
+        <is>
+          <t>Публичные лекции talks.cam</t>
+        </is>
+      </c>
+      <c r="C7" s="21" t="inlineStr">
+        <is>
+          <t>постоянно</t>
+        </is>
+      </c>
+      <c r="D7" s="21" t="inlineStr">
+        <is>
+          <t>S047, списки Major Public Lectures, Darwin College и др.</t>
+        </is>
+      </c>
+      <c r="E7" s="21" t="inlineStr">
+        <is>
+          <t>S047</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="21" t="inlineStr">
+        <is>
+          <t>C7</t>
+        </is>
+      </c>
+      <c r="B8" s="21" t="inlineStr">
+        <is>
+          <t>Открытия на Mill Road: Catte Latte, Hungarian Soul</t>
+        </is>
+      </c>
+      <c r="C8" s="21" t="inlineStr">
+        <is>
+          <t>уже прошли (архив)</t>
+        </is>
+      </c>
+      <c r="D8" s="21" t="inlineStr">
+        <is>
+          <t>Cambridge Foodies — поток «новое в городе»</t>
+        </is>
+      </c>
+      <c r="E8" s="21" t="inlineStr">
+        <is>
+          <t>Catte Latte, Hungarian Soul</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="21" t="inlineStr">
+        <is>
+          <t>C8</t>
+        </is>
+      </c>
+      <c r="B9" s="21" t="inlineStr">
+        <is>
+          <t>Cambridge Oktoberfest, Jesus Green</t>
+        </is>
+      </c>
+      <c r="C9" s="21" t="inlineStr">
+        <is>
+          <t>2026-09-25 – 2026-09-26</t>
+        </is>
+      </c>
+      <c r="D9" s="21" t="inlineStr">
+        <is>
+          <t>Eventbrite / Skiddle / Ents24 / Cambridge 105 / новости, если ещё видно</t>
+        </is>
+      </c>
+      <c r="E9" s="21" t="inlineStr">
+        <is>
+          <t>Oktoberfest</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7650,534 +8205,534 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="11">
-      <c r="A1" s="23" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t>Категория</t>
         </is>
       </c>
-      <c r="B1" s="23" t="inlineStr">
+      <c r="B1" s="25" t="inlineStr">
         <is>
           <t>Всего источников</t>
         </is>
       </c>
-      <c r="C1" s="23" t="inlineStr">
+      <c r="C1" s="25" t="inlineStr">
         <is>
           <t>Приоритет 1</t>
         </is>
       </c>
-      <c r="D1" s="23" t="inlineStr">
+      <c r="D1" s="25" t="inlineStr">
         <is>
           <t>URL проверен</t>
         </is>
       </c>
-      <c r="E1" s="23" t="inlineStr">
+      <c r="E1" s="25" t="inlineStr">
         <is>
           <t>Осталось проверить</t>
         </is>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="11">
-      <c r="A2" s="24" t="inlineStr">
+      <c r="A2" s="26" t="inlineStr">
         <is>
           <t>Сквозные агрегаторы</t>
         </is>
       </c>
-      <c r="B2" s="24">
-        <f>COUNTIF(Источники!$B$2:$B$90,A2)</f>
+      <c r="B2" s="26">
+        <f>COUNTIF(Источники!$B$2:$B$500,A2)</f>
         <v/>
       </c>
-      <c r="C2" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A2,Источники!$J$2:$J$90,1)</f>
+      <c r="C2" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A2,Источники!$J$2:$J$500,1)</f>
         <v/>
       </c>
-      <c r="D2" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A2,Источники!$K$2:$K$90,"да")</f>
+      <c r="D2" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A2,Источники!$K$2:$K$500,"да")</f>
         <v/>
       </c>
-      <c r="E2" s="24">
+      <c r="E2" s="26">
         <f>B2-D2</f>
         <v/>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="11">
-      <c r="A3" s="24" t="inlineStr">
+      <c r="A3" s="26" t="inlineStr">
         <is>
           <t>Концерты</t>
         </is>
       </c>
-      <c r="B3" s="24">
-        <f>COUNTIF(Источники!$B$2:$B$90,A3)</f>
+      <c r="B3" s="26">
+        <f>COUNTIF(Источники!$B$2:$B$500,A3)</f>
         <v/>
       </c>
-      <c r="C3" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A3,Источники!$J$2:$J$90,1)</f>
+      <c r="C3" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A3,Источники!$J$2:$J$500,1)</f>
         <v/>
       </c>
-      <c r="D3" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A3,Источники!$K$2:$K$90,"да")</f>
+      <c r="D3" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A3,Источники!$K$2:$K$500,"да")</f>
         <v/>
       </c>
-      <c r="E3" s="24">
+      <c r="E3" s="26">
         <f>B3-D3</f>
         <v/>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="11">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="26" t="inlineStr">
         <is>
           <t>Спорт — смотреть</t>
         </is>
       </c>
-      <c r="B4" s="24">
-        <f>COUNTIF(Источники!$B$2:$B$90,A4)</f>
+      <c r="B4" s="26">
+        <f>COUNTIF(Источники!$B$2:$B$500,A4)</f>
         <v/>
       </c>
-      <c r="C4" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A4,Источники!$J$2:$J$90,1)</f>
+      <c r="C4" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A4,Источники!$J$2:$J$500,1)</f>
         <v/>
       </c>
-      <c r="D4" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A4,Источники!$K$2:$K$90,"да")</f>
+      <c r="D4" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A4,Источники!$K$2:$K$500,"да")</f>
         <v/>
       </c>
-      <c r="E4" s="24">
+      <c r="E4" s="26">
         <f>B4-D4</f>
         <v/>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="11">
-      <c r="A5" s="24" t="inlineStr">
+      <c r="A5" s="26" t="inlineStr">
         <is>
           <t>Спорт — участвовать</t>
         </is>
       </c>
-      <c r="B5" s="24">
-        <f>COUNTIF(Источники!$B$2:$B$90,A5)</f>
+      <c r="B5" s="26">
+        <f>COUNTIF(Источники!$B$2:$B$500,A5)</f>
         <v/>
       </c>
-      <c r="C5" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A5,Источники!$J$2:$J$90,1)</f>
+      <c r="C5" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A5,Источники!$J$2:$J$500,1)</f>
         <v/>
       </c>
-      <c r="D5" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A5,Источники!$K$2:$K$90,"да")</f>
+      <c r="D5" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A5,Источники!$K$2:$K$500,"да")</f>
         <v/>
       </c>
-      <c r="E5" s="24">
+      <c r="E5" s="26">
         <f>B5-D5</f>
         <v/>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="11">
-      <c r="A6" s="24" t="inlineStr">
+      <c r="A6" s="26" t="inlineStr">
         <is>
           <t>Фестивали</t>
         </is>
       </c>
-      <c r="B6" s="24">
-        <f>COUNTIF(Источники!$B$2:$B$90,A6)</f>
+      <c r="B6" s="26">
+        <f>COUNTIF(Источники!$B$2:$B$500,A6)</f>
         <v/>
       </c>
-      <c r="C6" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A6,Источники!$J$2:$J$90,1)</f>
+      <c r="C6" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A6,Источники!$J$2:$J$500,1)</f>
         <v/>
       </c>
-      <c r="D6" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A6,Источники!$K$2:$K$90,"да")</f>
+      <c r="D6" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A6,Источники!$K$2:$K$500,"да")</f>
         <v/>
       </c>
-      <c r="E6" s="24">
+      <c r="E6" s="26">
         <f>B6-D6</f>
         <v/>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="11">
-      <c r="A7" s="24" t="inlineStr">
+      <c r="A7" s="26" t="inlineStr">
         <is>
           <t>Ярмарки</t>
         </is>
       </c>
-      <c r="B7" s="24">
-        <f>COUNTIF(Источники!$B$2:$B$90,A7)</f>
+      <c r="B7" s="26">
+        <f>COUNTIF(Источники!$B$2:$B$500,A7)</f>
         <v/>
       </c>
-      <c r="C7" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A7,Источники!$J$2:$J$90,1)</f>
+      <c r="C7" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A7,Источники!$J$2:$J$500,1)</f>
         <v/>
       </c>
-      <c r="D7" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A7,Источники!$K$2:$K$90,"да")</f>
+      <c r="D7" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A7,Источники!$K$2:$K$500,"да")</f>
         <v/>
       </c>
-      <c r="E7" s="24">
+      <c r="E7" s="26">
         <f>B7-D7</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="11">
-      <c r="A8" s="24" t="inlineStr">
+      <c r="A8" s="26" t="inlineStr">
         <is>
           <t>Театр</t>
         </is>
       </c>
-      <c r="B8" s="24">
-        <f>COUNTIF(Источники!$B$2:$B$90,A8)</f>
+      <c r="B8" s="26">
+        <f>COUNTIF(Источники!$B$2:$B$500,A8)</f>
         <v/>
       </c>
-      <c r="C8" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A8,Источники!$J$2:$J$90,1)</f>
+      <c r="C8" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A8,Источники!$J$2:$J$500,1)</f>
         <v/>
       </c>
-      <c r="D8" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A8,Источники!$K$2:$K$90,"да")</f>
+      <c r="D8" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A8,Источники!$K$2:$K$500,"да")</f>
         <v/>
       </c>
-      <c r="E8" s="24">
+      <c r="E8" s="26">
         <f>B8-D8</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="11">
-      <c r="A9" s="24" t="inlineStr">
+      <c r="A9" s="26" t="inlineStr">
         <is>
           <t>Кино</t>
         </is>
       </c>
-      <c r="B9" s="24">
-        <f>COUNTIF(Источники!$B$2:$B$90,A9)</f>
+      <c r="B9" s="26">
+        <f>COUNTIF(Источники!$B$2:$B$500,A9)</f>
         <v/>
       </c>
-      <c r="C9" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A9,Источники!$J$2:$J$90,1)</f>
+      <c r="C9" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A9,Источники!$J$2:$J$500,1)</f>
         <v/>
       </c>
-      <c r="D9" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A9,Источники!$K$2:$K$90,"да")</f>
+      <c r="D9" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A9,Источники!$K$2:$K$500,"да")</f>
         <v/>
       </c>
-      <c r="E9" s="24">
+      <c r="E9" s="26">
         <f>B9-D9</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="11">
-      <c r="A10" s="24" t="inlineStr">
+      <c r="A10" s="26" t="inlineStr">
         <is>
           <t>Лекции</t>
         </is>
       </c>
-      <c r="B10" s="24">
-        <f>COUNTIF(Источники!$B$2:$B$90,A10)</f>
+      <c r="B10" s="26">
+        <f>COUNTIF(Источники!$B$2:$B$500,A10)</f>
         <v/>
       </c>
-      <c r="C10" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A10,Источники!$J$2:$J$90,1)</f>
+      <c r="C10" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A10,Источники!$J$2:$J$500,1)</f>
         <v/>
       </c>
-      <c r="D10" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A10,Источники!$K$2:$K$90,"да")</f>
+      <c r="D10" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A10,Источники!$K$2:$K$500,"да")</f>
         <v/>
       </c>
-      <c r="E10" s="24">
+      <c r="E10" s="26">
         <f>B10-D10</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="11">
-      <c r="A11" s="24" t="inlineStr">
+      <c r="A11" s="26" t="inlineStr">
         <is>
           <t>Выставки и музеи</t>
         </is>
       </c>
-      <c r="B11" s="24">
-        <f>COUNTIF(Источники!$B$2:$B$90,A11)</f>
+      <c r="B11" s="26">
+        <f>COUNTIF(Источники!$B$2:$B$500,A11)</f>
         <v/>
       </c>
-      <c r="C11" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A11,Источники!$J$2:$J$90,1)</f>
+      <c r="C11" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A11,Источники!$J$2:$J$500,1)</f>
         <v/>
       </c>
-      <c r="D11" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A11,Источники!$K$2:$K$90,"да")</f>
+      <c r="D11" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A11,Источники!$K$2:$K$500,"да")</f>
         <v/>
       </c>
-      <c r="E11" s="24">
+      <c r="E11" s="26">
         <f>B11-D11</f>
         <v/>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="11">
-      <c r="A12" s="24" t="inlineStr">
+      <c r="A12" s="26" t="inlineStr">
         <is>
           <t>Детям и семьям</t>
         </is>
       </c>
-      <c r="B12" s="24">
-        <f>COUNTIF(Источники!$B$2:$B$90,A12)</f>
+      <c r="B12" s="26">
+        <f>COUNTIF(Источники!$B$2:$B$500,A12)</f>
         <v/>
       </c>
-      <c r="C12" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A12,Источники!$J$2:$J$90,1)</f>
+      <c r="C12" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A12,Источники!$J$2:$J$500,1)</f>
         <v/>
       </c>
-      <c r="D12" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A12,Источники!$K$2:$K$90,"да")</f>
+      <c r="D12" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A12,Источники!$K$2:$K$500,"да")</f>
         <v/>
       </c>
-      <c r="E12" s="24">
+      <c r="E12" s="26">
         <f>B12-D12</f>
         <v/>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="11">
-      <c r="A13" s="24" t="inlineStr">
+      <c r="A13" s="26" t="inlineStr">
         <is>
           <t>Еда и напитки</t>
         </is>
       </c>
-      <c r="B13" s="24">
-        <f>COUNTIF(Источники!$B$2:$B$90,A13)</f>
+      <c r="B13" s="26">
+        <f>COUNTIF(Источники!$B$2:$B$500,A13)</f>
         <v/>
       </c>
-      <c r="C13" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A13,Источники!$J$2:$J$90,1)</f>
+      <c r="C13" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A13,Источники!$J$2:$J$500,1)</f>
         <v/>
       </c>
-      <c r="D13" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A13,Источники!$K$2:$K$90,"да")</f>
+      <c r="D13" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A13,Источники!$K$2:$K$500,"да")</f>
         <v/>
       </c>
-      <c r="E13" s="24">
+      <c r="E13" s="26">
         <f>B13-D13</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="11">
-      <c r="A14" s="24" t="inlineStr">
+      <c r="A14" s="26" t="inlineStr">
         <is>
           <t>Рынки и барахолки</t>
         </is>
       </c>
-      <c r="B14" s="24">
-        <f>COUNTIF(Источники!$B$2:$B$90,A14)</f>
+      <c r="B14" s="26">
+        <f>COUNTIF(Источники!$B$2:$B$500,A14)</f>
         <v/>
       </c>
-      <c r="C14" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A14,Источники!$J$2:$J$90,1)</f>
+      <c r="C14" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A14,Источники!$J$2:$J$500,1)</f>
         <v/>
       </c>
-      <c r="D14" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A14,Источники!$K$2:$K$90,"да")</f>
+      <c r="D14" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A14,Источники!$K$2:$K$500,"да")</f>
         <v/>
       </c>
-      <c r="E14" s="24">
+      <c r="E14" s="26">
         <f>B14-D14</f>
         <v/>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="11">
-      <c r="A15" s="24" t="inlineStr">
+      <c r="A15" s="26" t="inlineStr">
         <is>
           <t>Комедия и стендап</t>
         </is>
       </c>
-      <c r="B15" s="24">
-        <f>COUNTIF(Источники!$B$2:$B$90,A15)</f>
+      <c r="B15" s="26">
+        <f>COUNTIF(Источники!$B$2:$B$500,A15)</f>
         <v/>
       </c>
-      <c r="C15" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A15,Источники!$J$2:$J$90,1)</f>
+      <c r="C15" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A15,Источники!$J$2:$J$500,1)</f>
         <v/>
       </c>
-      <c r="D15" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A15,Источники!$K$2:$K$90,"да")</f>
+      <c r="D15" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A15,Источники!$K$2:$K$500,"да")</f>
         <v/>
       </c>
-      <c r="E15" s="24">
+      <c r="E15" s="26">
         <f>B15-D15</f>
         <v/>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="11">
-      <c r="A16" s="24" t="inlineStr">
+      <c r="A16" s="26" t="inlineStr">
         <is>
           <t>Ночная жизнь</t>
         </is>
       </c>
-      <c r="B16" s="24">
-        <f>COUNTIF(Источники!$B$2:$B$90,A16)</f>
+      <c r="B16" s="26">
+        <f>COUNTIF(Источники!$B$2:$B$500,A16)</f>
         <v/>
       </c>
-      <c r="C16" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A16,Источники!$J$2:$J$90,1)</f>
+      <c r="C16" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A16,Источники!$J$2:$J$500,1)</f>
         <v/>
       </c>
-      <c r="D16" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A16,Источники!$K$2:$K$90,"да")</f>
+      <c r="D16" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A16,Источники!$K$2:$K$500,"да")</f>
         <v/>
       </c>
-      <c r="E16" s="24">
+      <c r="E16" s="26">
         <f>B16-D16</f>
         <v/>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="11">
-      <c r="A17" s="24" t="inlineStr">
+      <c r="A17" s="26" t="inlineStr">
         <is>
           <t>Открытые двери и экскурсии</t>
         </is>
       </c>
-      <c r="B17" s="24">
-        <f>COUNTIF(Источники!$B$2:$B$90,A17)</f>
+      <c r="B17" s="26">
+        <f>COUNTIF(Источники!$B$2:$B$500,A17)</f>
         <v/>
       </c>
-      <c r="C17" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A17,Источники!$J$2:$J$90,1)</f>
+      <c r="C17" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A17,Источники!$J$2:$J$500,1)</f>
         <v/>
       </c>
-      <c r="D17" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A17,Источники!$K$2:$K$90,"да")</f>
+      <c r="D17" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A17,Источники!$K$2:$K$500,"да")</f>
         <v/>
       </c>
-      <c r="E17" s="24">
+      <c r="E17" s="26">
         <f>B17-D17</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="11">
-      <c r="A18" s="24" t="inlineStr">
+      <c r="A18" s="26" t="inlineStr">
         <is>
           <t>Природа и загородные поездки</t>
         </is>
       </c>
-      <c r="B18" s="24">
-        <f>COUNTIF(Источники!$B$2:$B$90,A18)</f>
+      <c r="B18" s="26">
+        <f>COUNTIF(Источники!$B$2:$B$500,A18)</f>
         <v/>
       </c>
-      <c r="C18" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A18,Источники!$J$2:$J$90,1)</f>
+      <c r="C18" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A18,Источники!$J$2:$J$500,1)</f>
         <v/>
       </c>
-      <c r="D18" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A18,Источники!$K$2:$K$90,"да")</f>
+      <c r="D18" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A18,Источники!$K$2:$K$500,"да")</f>
         <v/>
       </c>
-      <c r="E18" s="24">
+      <c r="E18" s="26">
         <f>B18-D18</f>
         <v/>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="11">
-      <c r="A19" s="24" t="inlineStr">
+      <c r="A19" s="26" t="inlineStr">
         <is>
           <t>Праздники и сезонное</t>
         </is>
       </c>
-      <c r="B19" s="24">
-        <f>COUNTIF(Источники!$B$2:$B$90,A19)</f>
+      <c r="B19" s="26">
+        <f>COUNTIF(Источники!$B$2:$B$500,A19)</f>
         <v/>
       </c>
-      <c r="C19" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A19,Источники!$J$2:$J$90,1)</f>
+      <c r="C19" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A19,Источники!$J$2:$J$500,1)</f>
         <v/>
       </c>
-      <c r="D19" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A19,Источники!$K$2:$K$90,"да")</f>
+      <c r="D19" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A19,Источники!$K$2:$K$500,"да")</f>
         <v/>
       </c>
-      <c r="E19" s="24">
+      <c r="E19" s="26">
         <f>B19-D19</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="11">
-      <c r="A20" s="24" t="inlineStr">
+      <c r="A20" s="26" t="inlineStr">
         <is>
           <t>Воркшопы и курсы</t>
         </is>
       </c>
-      <c r="B20" s="24">
-        <f>COUNTIF(Источники!$B$2:$B$90,A20)</f>
+      <c r="B20" s="26">
+        <f>COUNTIF(Источники!$B$2:$B$500,A20)</f>
         <v/>
       </c>
-      <c r="C20" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A20,Источники!$J$2:$J$90,1)</f>
+      <c r="C20" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A20,Источники!$J$2:$J$500,1)</f>
         <v/>
       </c>
-      <c r="D20" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A20,Источники!$K$2:$K$90,"да")</f>
+      <c r="D20" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A20,Источники!$K$2:$K$500,"да")</f>
         <v/>
       </c>
-      <c r="E20" s="24">
+      <c r="E20" s="26">
         <f>B20-D20</f>
         <v/>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="11">
-      <c r="A21" s="24" t="inlineStr">
+      <c r="A21" s="26" t="inlineStr">
         <is>
           <t>Сообщества и благотворительность</t>
         </is>
       </c>
-      <c r="B21" s="24">
-        <f>COUNTIF(Источники!$B$2:$B$90,A21)</f>
+      <c r="B21" s="26">
+        <f>COUNTIF(Источники!$B$2:$B$500,A21)</f>
         <v/>
       </c>
-      <c r="C21" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A21,Источники!$J$2:$J$90,1)</f>
+      <c r="C21" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A21,Источники!$J$2:$J$500,1)</f>
         <v/>
       </c>
-      <c r="D21" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A21,Источники!$K$2:$K$90,"да")</f>
+      <c r="D21" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A21,Источники!$K$2:$K$500,"да")</f>
         <v/>
       </c>
-      <c r="E21" s="24">
+      <c r="E21" s="26">
         <f>B21-D21</f>
         <v/>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="11">
-      <c r="A22" s="24" t="inlineStr">
+      <c r="A22" s="26" t="inlineStr">
         <is>
           <t>Практическое</t>
         </is>
       </c>
-      <c r="B22" s="24">
-        <f>COUNTIF(Источники!$B$2:$B$90,A22)</f>
+      <c r="B22" s="26">
+        <f>COUNTIF(Источники!$B$2:$B$500,A22)</f>
         <v/>
       </c>
-      <c r="C22" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A22,Источники!$J$2:$J$90,1)</f>
+      <c r="C22" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A22,Источники!$J$2:$J$500,1)</f>
         <v/>
       </c>
-      <c r="D22" s="24">
-        <f>COUNTIFS(Источники!$B$2:$B$90,A22,Источники!$K$2:$K$90,"да")</f>
+      <c r="D22" s="26">
+        <f>COUNTIFS(Источники!$B$2:$B$500,A22,Источники!$K$2:$K$500,"да")</f>
         <v/>
       </c>
-      <c r="E22" s="24">
+      <c r="E22" s="26">
         <f>B22-D22</f>
         <v/>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="11">
-      <c r="A23" s="25" t="inlineStr">
+      <c r="A23" s="27" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
       </c>
-      <c r="B23" s="25">
+      <c r="B23" s="27">
         <f>SUM(B2:B22)</f>
         <v/>
       </c>
-      <c r="C23" s="25">
+      <c r="C23" s="27">
         <f>SUM(C2:C22)</f>
         <v/>
       </c>
-      <c r="D23" s="25">
+      <c r="D23" s="27">
         <f>SUM(D2:D22)</f>
         <v/>
       </c>
-      <c r="E23" s="25">
+      <c r="E23" s="27">
         <f>SUM(E2:E22)</f>
         <v/>
       </c>
@@ -8189,7 +8744,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8206,604 +8761,604 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="11">
-      <c r="A1" s="23" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t>Поле</t>
         </is>
       </c>
-      <c r="B1" s="23" t="inlineStr">
+      <c r="B1" s="25" t="inlineStr">
         <is>
           <t>Тип</t>
         </is>
       </c>
-      <c r="C1" s="23" t="inlineStr">
+      <c r="C1" s="25" t="inlineStr">
         <is>
           <t>Обязательное</t>
         </is>
       </c>
-      <c r="D1" s="23" t="inlineStr">
+      <c r="D1" s="25" t="inlineStr">
         <is>
           <t>Пример</t>
         </is>
       </c>
-      <c r="E1" s="23" t="inlineStr">
+      <c r="E1" s="25" t="inlineStr">
         <is>
           <t>Комментарий</t>
         </is>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="11">
-      <c r="A2" s="26" t="inlineStr">
+      <c r="A2" s="28" t="inlineStr">
         <is>
           <t>event_id</t>
         </is>
       </c>
-      <c r="B2" s="26" t="inlineStr">
+      <c r="B2" s="28" t="inlineStr">
         <is>
           <t>текст</t>
         </is>
       </c>
-      <c r="C2" s="26" t="inlineStr">
+      <c r="C2" s="28" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D2" s="26" t="inlineStr">
+      <c r="D2" s="28" t="inlineStr">
         <is>
           <t>EV-2026-000123</t>
         </is>
       </c>
-      <c r="E2" s="26" t="inlineStr">
+      <c r="E2" s="28" t="inlineStr">
         <is>
           <t>Внутренний ID</t>
         </is>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="11">
-      <c r="A3" s="26" t="inlineStr">
+      <c r="A3" s="28" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="B3" s="26" t="inlineStr">
+      <c r="B3" s="28" t="inlineStr">
         <is>
           <t>текст</t>
         </is>
       </c>
-      <c r="C3" s="26" t="inlineStr">
+      <c r="C3" s="28" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D3" s="26" t="inlineStr">
+      <c r="D3" s="28" t="inlineStr">
         <is>
           <t>Cambridge United vs AFC Wimbledon</t>
         </is>
       </c>
-      <c r="E3" s="26" t="n"/>
+      <c r="E3" s="28" t="n"/>
     </row>
     <row r="4" ht="15" customHeight="1" s="11">
-      <c r="A4" s="26" t="inlineStr">
+      <c r="A4" s="28" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="B4" s="26" t="inlineStr">
+      <c r="B4" s="28" t="inlineStr">
         <is>
           <t>список</t>
         </is>
       </c>
-      <c r="C4" s="26" t="inlineStr">
+      <c r="C4" s="28" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D4" s="26" t="inlineStr">
+      <c r="D4" s="28" t="inlineStr">
         <is>
           <t>Спорт — смотреть</t>
         </is>
       </c>
-      <c r="E4" s="26" t="inlineStr">
+      <c r="E4" s="28" t="inlineStr">
         <is>
           <t>Из листа «Категории и теги»</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="11">
-      <c r="A5" s="26" t="inlineStr">
+      <c r="A5" s="28" t="inlineStr">
         <is>
           <t>date_start</t>
         </is>
       </c>
-      <c r="B5" s="26" t="inlineStr">
+      <c r="B5" s="28" t="inlineStr">
         <is>
           <t>дата</t>
         </is>
       </c>
-      <c r="C5" s="26" t="inlineStr">
+      <c r="C5" s="28" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D5" s="26" t="inlineStr">
+      <c r="D5" s="28" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="E5" s="26" t="n"/>
+      <c r="E5" s="28" t="n"/>
     </row>
     <row r="6" ht="15" customHeight="1" s="11">
-      <c r="A6" s="26" t="inlineStr">
+      <c r="A6" s="28" t="inlineStr">
         <is>
           <t>time_start</t>
         </is>
       </c>
-      <c r="B6" s="26" t="inlineStr">
+      <c r="B6" s="28" t="inlineStr">
         <is>
           <t>время</t>
         </is>
       </c>
-      <c r="C6" s="26" t="inlineStr">
+      <c r="C6" s="28" t="inlineStr">
         <is>
           <t>да, если известно</t>
         </is>
       </c>
-      <c r="D6" s="26" t="inlineStr">
+      <c r="D6" s="28" t="inlineStr">
         <is>
           <t>15:00</t>
         </is>
       </c>
-      <c r="E6" s="26" t="inlineStr">
+      <c r="E6" s="28" t="inlineStr">
         <is>
           <t>Пусто = весь день</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="11">
-      <c r="A7" s="26" t="inlineStr">
+      <c r="A7" s="28" t="inlineStr">
         <is>
           <t>date_end</t>
         </is>
       </c>
-      <c r="B7" s="26" t="inlineStr">
+      <c r="B7" s="28" t="inlineStr">
         <is>
           <t>дата</t>
         </is>
       </c>
-      <c r="C7" s="26" t="inlineStr">
+      <c r="C7" s="28" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
-      <c r="D7" s="26" t="inlineStr">
+      <c r="D7" s="28" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="E7" s="26" t="inlineStr">
+      <c r="E7" s="28" t="inlineStr">
         <is>
           <t>Для многодневных</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="11">
-      <c r="A8" s="26" t="inlineStr">
+      <c r="A8" s="28" t="inlineStr">
         <is>
           <t>time_end</t>
         </is>
       </c>
-      <c r="B8" s="26" t="inlineStr">
+      <c r="B8" s="28" t="inlineStr">
         <is>
           <t>время</t>
         </is>
       </c>
-      <c r="C8" s="26" t="inlineStr">
+      <c r="C8" s="28" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
-      <c r="D8" s="26" t="inlineStr">
+      <c r="D8" s="28" t="inlineStr">
         <is>
           <t>17:00</t>
         </is>
       </c>
-      <c r="E8" s="26" t="n"/>
+      <c r="E8" s="28" t="n"/>
     </row>
     <row r="9" ht="15" customHeight="1" s="11">
-      <c r="A9" s="26" t="inlineStr">
+      <c r="A9" s="28" t="inlineStr">
         <is>
           <t>venue_name</t>
         </is>
       </c>
-      <c r="B9" s="26" t="inlineStr">
+      <c r="B9" s="28" t="inlineStr">
         <is>
           <t>текст</t>
         </is>
       </c>
-      <c r="C9" s="26" t="inlineStr">
+      <c r="C9" s="28" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D9" s="26" t="inlineStr">
+      <c r="D9" s="28" t="inlineStr">
         <is>
           <t>Abbey Stadium</t>
         </is>
       </c>
-      <c r="E9" s="26" t="n"/>
+      <c r="E9" s="28" t="n"/>
     </row>
     <row r="10" ht="15" customHeight="1" s="11">
-      <c r="A10" s="26" t="inlineStr">
+      <c r="A10" s="28" t="inlineStr">
         <is>
           <t>address</t>
         </is>
       </c>
-      <c r="B10" s="26" t="inlineStr">
+      <c r="B10" s="28" t="inlineStr">
         <is>
           <t>текст</t>
         </is>
       </c>
-      <c r="C10" s="26" t="inlineStr">
+      <c r="C10" s="28" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D10" s="26" t="inlineStr">
+      <c r="D10" s="28" t="inlineStr">
         <is>
           <t>Newmarket Road, Cambridge</t>
         </is>
       </c>
-      <c r="E10" s="26" t="inlineStr">
+      <c r="E10" s="28" t="inlineStr">
         <is>
           <t>Точный адрес</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="11">
-      <c r="A11" s="26" t="inlineStr">
+      <c r="A11" s="28" t="inlineStr">
         <is>
           <t>postcode</t>
         </is>
       </c>
-      <c r="B11" s="26" t="inlineStr">
+      <c r="B11" s="28" t="inlineStr">
         <is>
           <t>текст</t>
         </is>
       </c>
-      <c r="C11" s="26" t="inlineStr">
+      <c r="C11" s="28" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D11" s="26" t="inlineStr">
+      <c r="D11" s="28" t="inlineStr">
         <is>
           <t>(заполнять из источника)</t>
         </is>
       </c>
-      <c r="E11" s="26" t="inlineStr">
+      <c r="E11" s="28" t="inlineStr">
         <is>
           <t>Для карты и расчёта зоны</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="11">
-      <c r="A12" s="26" t="inlineStr">
+      <c r="A12" s="28" t="inlineStr">
         <is>
           <t>lat / lon</t>
         </is>
       </c>
-      <c r="B12" s="26" t="inlineStr">
+      <c r="B12" s="28" t="inlineStr">
         <is>
           <t>число</t>
         </is>
       </c>
-      <c r="C12" s="26" t="inlineStr">
+      <c r="C12" s="28" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
-      <c r="D12" s="26" t="inlineStr">
+      <c r="D12" s="28" t="inlineStr">
         <is>
           <t>52.21, 0.15</t>
         </is>
       </c>
-      <c r="E12" s="26" t="inlineStr">
+      <c r="E12" s="28" t="inlineStr">
         <is>
           <t>Геокодирование по postcode</t>
         </is>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="11">
-      <c r="A13" s="26" t="inlineStr">
+      <c r="A13" s="28" t="inlineStr">
         <is>
           <t>zone</t>
         </is>
       </c>
-      <c r="B13" s="26" t="inlineStr">
+      <c r="B13" s="28" t="inlineStr">
         <is>
           <t>список</t>
         </is>
       </c>
-      <c r="C13" s="26" t="inlineStr">
+      <c r="C13" s="28" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D13" s="26" t="inlineStr">
+      <c r="D13" s="28" t="inlineStr">
         <is>
           <t>Центр</t>
         </is>
       </c>
-      <c r="E13" s="26" t="inlineStr">
+      <c r="E13" s="28" t="inlineStr">
         <is>
           <t>Тег: Центр / до 30 мин / до часа — считается автоматически</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="11">
-      <c r="A14" s="26" t="inlineStr">
+      <c r="A14" s="28" t="inlineStr">
         <is>
           <t>price_from</t>
         </is>
       </c>
-      <c r="B14" s="26" t="inlineStr">
+      <c r="B14" s="28" t="inlineStr">
         <is>
           <t>число, £</t>
         </is>
       </c>
-      <c r="C14" s="26" t="inlineStr">
+      <c r="C14" s="28" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
-      <c r="D14" s="26" t="inlineStr">
+      <c r="D14" s="28" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="E14" s="26" t="inlineStr">
+      <c r="E14" s="28" t="inlineStr">
         <is>
           <t>0 = бесплатно</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="11">
-      <c r="A15" s="26" t="inlineStr">
+      <c r="A15" s="28" t="inlineStr">
         <is>
           <t>price_tag</t>
         </is>
       </c>
-      <c r="B15" s="26" t="inlineStr">
+      <c r="B15" s="28" t="inlineStr">
         <is>
           <t>список</t>
         </is>
       </c>
-      <c r="C15" s="26" t="inlineStr">
+      <c r="C15" s="28" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D15" s="26" t="inlineStr">
+      <c r="D15" s="28" t="inlineStr">
         <is>
           <t>бесплатно / до £10 / дороже</t>
         </is>
       </c>
-      <c r="E15" s="26" t="n"/>
+      <c r="E15" s="28" t="n"/>
     </row>
     <row r="16" ht="15" customHeight="1" s="11">
-      <c r="A16" s="26" t="inlineStr">
+      <c r="A16" s="28" t="inlineStr">
         <is>
           <t>audience</t>
         </is>
       </c>
-      <c r="B16" s="26" t="inlineStr">
+      <c r="B16" s="28" t="inlineStr">
         <is>
           <t>список (несколько)</t>
         </is>
       </c>
-      <c r="C16" s="26" t="inlineStr">
+      <c r="C16" s="28" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
-      <c r="D16" s="26" t="inlineStr">
+      <c r="D16" s="28" t="inlineStr">
         <is>
           <t>дети 5–12; семьи</t>
         </is>
       </c>
-      <c r="E16" s="26" t="n"/>
+      <c r="E16" s="28" t="n"/>
     </row>
     <row r="17" ht="23.85" customHeight="1" s="11">
-      <c r="A17" s="26" t="inlineStr">
+      <c r="A17" s="28" t="inlineStr">
         <is>
           <t>booking</t>
         </is>
       </c>
-      <c r="B17" s="26" t="inlineStr">
+      <c r="B17" s="28" t="inlineStr">
         <is>
           <t>список</t>
         </is>
       </c>
-      <c r="C17" s="26" t="inlineStr">
+      <c r="C17" s="28" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D17" s="26" t="inlineStr">
+      <c r="D17" s="28" t="inlineStr">
         <is>
           <t>без билетов / бронировать / продажа скоро</t>
         </is>
       </c>
-      <c r="E17" s="26" t="n"/>
+      <c r="E17" s="28" t="n"/>
     </row>
     <row r="18" ht="15" customHeight="1" s="11">
-      <c r="A18" s="26" t="inlineStr">
+      <c r="A18" s="28" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="B18" s="26" t="inlineStr">
+      <c r="B18" s="28" t="inlineStr">
         <is>
           <t>список</t>
         </is>
       </c>
-      <c r="C18" s="26" t="inlineStr">
+      <c r="C18" s="28" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D18" s="26" t="inlineStr">
+      <c r="D18" s="28" t="inlineStr">
         <is>
           <t>по плану</t>
         </is>
       </c>
-      <c r="E18" s="26" t="inlineStr">
+      <c r="E18" s="28" t="inlineStr">
         <is>
           <t>по плану / перенесено / отменено / sold out</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="11">
-      <c r="A19" s="26" t="inlineStr">
+      <c r="A19" s="28" t="inlineStr">
         <is>
           <t>ticket_url</t>
         </is>
       </c>
-      <c r="B19" s="26" t="inlineStr">
+      <c r="B19" s="28" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
       </c>
-      <c r="C19" s="26" t="inlineStr">
+      <c r="C19" s="28" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
-      <c r="D19" s="26" t="n"/>
-      <c r="E19" s="26" t="inlineStr">
+      <c r="D19" s="28" t="n"/>
+      <c r="E19" s="28" t="inlineStr">
         <is>
           <t>Здесь партнёрская ссылка, если есть</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="11">
-      <c r="A20" s="26" t="inlineStr">
+      <c r="A20" s="28" t="inlineStr">
         <is>
           <t>source_id</t>
         </is>
       </c>
-      <c r="B20" s="26" t="inlineStr">
+      <c r="B20" s="28" t="inlineStr">
         <is>
           <t>ссылка</t>
         </is>
       </c>
-      <c r="C20" s="26" t="inlineStr">
+      <c r="C20" s="28" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D20" s="26" t="inlineStr">
+      <c r="D20" s="28" t="inlineStr">
         <is>
           <t>S018</t>
         </is>
       </c>
-      <c r="E20" s="26" t="inlineStr">
+      <c r="E20" s="28" t="inlineStr">
         <is>
           <t>ID из листа «Источники»</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="11">
-      <c r="A21" s="26" t="inlineStr">
+      <c r="A21" s="28" t="inlineStr">
         <is>
           <t>source_url</t>
         </is>
       </c>
-      <c r="B21" s="26" t="inlineStr">
+      <c r="B21" s="28" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
       </c>
-      <c r="C21" s="26" t="inlineStr">
+      <c r="C21" s="28" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D21" s="26" t="n"/>
-      <c r="E21" s="26" t="inlineStr">
+      <c r="D21" s="28" t="n"/>
+      <c r="E21" s="28" t="inlineStr">
         <is>
           <t>Страница события у первоисточника</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="11">
-      <c r="A22" s="26" t="inlineStr">
+      <c r="A22" s="28" t="inlineStr">
         <is>
           <t>description_short</t>
         </is>
       </c>
-      <c r="B22" s="26" t="inlineStr">
+      <c r="B22" s="28" t="inlineStr">
         <is>
           <t>текст</t>
         </is>
       </c>
-      <c r="C22" s="26" t="inlineStr">
+      <c r="C22" s="28" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D22" s="26" t="n"/>
-      <c r="E22" s="26" t="inlineStr">
+      <c r="D22" s="28" t="n"/>
+      <c r="E22" s="28" t="inlineStr">
         <is>
           <t>2–3 предложения своими словами (не копировать)</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="11">
-      <c r="A23" s="26" t="inlineStr">
+      <c r="A23" s="28" t="inlineStr">
         <is>
           <t>score</t>
         </is>
       </c>
-      <c r="B23" s="26" t="inlineStr">
+      <c r="B23" s="28" t="inlineStr">
         <is>
           <t>число 1–10</t>
         </is>
       </c>
-      <c r="C23" s="26" t="inlineStr">
+      <c r="C23" s="28" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
-      <c r="D23" s="26" t="inlineStr">
+      <c r="D23" s="28" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="E23" s="26" t="inlineStr">
+      <c r="E23" s="28" t="inlineStr">
         <is>
           <t>Оценка LLM «стоит ли внимания»</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="11">
-      <c r="A24" s="26" t="inlineStr">
+      <c r="A24" s="28" t="inlineStr">
         <is>
           <t>last_checked</t>
         </is>
       </c>
-      <c r="B24" s="26" t="inlineStr">
+      <c r="B24" s="28" t="inlineStr">
         <is>
           <t>дата-время</t>
         </is>
       </c>
-      <c r="C24" s="26" t="inlineStr">
+      <c r="C24" s="28" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D24" s="26" t="n"/>
-      <c r="E24" s="26" t="inlineStr">
+      <c r="D24" s="28" t="n"/>
+      <c r="E24" s="28" t="inlineStr">
         <is>
           <t>Когда контур отмен последний раз проверял</t>
         </is>
@@ -8816,7 +9371,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8830,468 +9385,468 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="11">
-      <c r="A1" s="23" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t>Ось</t>
         </is>
       </c>
-      <c r="B1" s="23" t="inlineStr">
+      <c r="B1" s="25" t="inlineStr">
         <is>
           <t>Значение</t>
         </is>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="11">
-      <c r="A2" s="24" t="inlineStr">
+      <c r="A2" s="26" t="inlineStr">
         <is>
           <t>Категория</t>
         </is>
       </c>
-      <c r="B2" s="24" t="inlineStr">
+      <c r="B2" s="26" t="inlineStr">
         <is>
           <t>Концерты</t>
         </is>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="11">
-      <c r="A3" s="24" t="inlineStr">
+      <c r="A3" s="26" t="inlineStr">
         <is>
           <t>Категория</t>
         </is>
       </c>
-      <c r="B3" s="24" t="inlineStr">
+      <c r="B3" s="26" t="inlineStr">
         <is>
           <t>Спорт — смотреть</t>
         </is>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="11">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="26" t="inlineStr">
         <is>
           <t>Категория</t>
         </is>
       </c>
-      <c r="B4" s="24" t="inlineStr">
+      <c r="B4" s="26" t="inlineStr">
         <is>
           <t>Спорт — участвовать</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="11">
-      <c r="A5" s="24" t="inlineStr">
+      <c r="A5" s="26" t="inlineStr">
         <is>
           <t>Категория</t>
         </is>
       </c>
-      <c r="B5" s="24" t="inlineStr">
+      <c r="B5" s="26" t="inlineStr">
         <is>
           <t>Фестивали</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="11">
-      <c r="A6" s="24" t="inlineStr">
+      <c r="A6" s="26" t="inlineStr">
         <is>
           <t>Категория</t>
         </is>
       </c>
-      <c r="B6" s="24" t="inlineStr">
+      <c r="B6" s="26" t="inlineStr">
         <is>
           <t>Ярмарки</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="11">
-      <c r="A7" s="24" t="inlineStr">
+      <c r="A7" s="26" t="inlineStr">
         <is>
           <t>Категория</t>
         </is>
       </c>
-      <c r="B7" s="24" t="inlineStr">
+      <c r="B7" s="26" t="inlineStr">
         <is>
           <t>Театр</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="11">
-      <c r="A8" s="24" t="inlineStr">
+      <c r="A8" s="26" t="inlineStr">
         <is>
           <t>Категория</t>
         </is>
       </c>
-      <c r="B8" s="24" t="inlineStr">
+      <c r="B8" s="26" t="inlineStr">
         <is>
           <t>Кино</t>
         </is>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="11">
-      <c r="A9" s="24" t="inlineStr">
+      <c r="A9" s="26" t="inlineStr">
         <is>
           <t>Категория</t>
         </is>
       </c>
-      <c r="B9" s="24" t="inlineStr">
+      <c r="B9" s="26" t="inlineStr">
         <is>
           <t>Лекции</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="11">
-      <c r="A10" s="24" t="inlineStr">
+      <c r="A10" s="26" t="inlineStr">
         <is>
           <t>Категория</t>
         </is>
       </c>
-      <c r="B10" s="24" t="inlineStr">
+      <c r="B10" s="26" t="inlineStr">
         <is>
           <t>Выставки и музеи</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="11">
-      <c r="A11" s="24" t="inlineStr">
+      <c r="A11" s="26" t="inlineStr">
         <is>
           <t>Категория</t>
         </is>
       </c>
-      <c r="B11" s="24" t="inlineStr">
+      <c r="B11" s="26" t="inlineStr">
         <is>
           <t>Детям и семьям</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="11">
-      <c r="A12" s="24" t="inlineStr">
+      <c r="A12" s="26" t="inlineStr">
         <is>
           <t>Категория</t>
         </is>
       </c>
-      <c r="B12" s="24" t="inlineStr">
+      <c r="B12" s="26" t="inlineStr">
         <is>
           <t>Еда и напитки</t>
         </is>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="11">
-      <c r="A13" s="24" t="inlineStr">
+      <c r="A13" s="26" t="inlineStr">
         <is>
           <t>Категория</t>
         </is>
       </c>
-      <c r="B13" s="24" t="inlineStr">
+      <c r="B13" s="26" t="inlineStr">
         <is>
           <t>Рынки и барахолки</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="11">
-      <c r="A14" s="24" t="inlineStr">
+      <c r="A14" s="26" t="inlineStr">
         <is>
           <t>Категория</t>
         </is>
       </c>
-      <c r="B14" s="24" t="inlineStr">
+      <c r="B14" s="26" t="inlineStr">
         <is>
           <t>Комедия и стендап</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="11">
-      <c r="A15" s="24" t="inlineStr">
+      <c r="A15" s="26" t="inlineStr">
         <is>
           <t>Категория</t>
         </is>
       </c>
-      <c r="B15" s="24" t="inlineStr">
+      <c r="B15" s="26" t="inlineStr">
         <is>
           <t>Ночная жизнь</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="11">
-      <c r="A16" s="24" t="inlineStr">
+      <c r="A16" s="26" t="inlineStr">
         <is>
           <t>Категория</t>
         </is>
       </c>
-      <c r="B16" s="24" t="inlineStr">
+      <c r="B16" s="26" t="inlineStr">
         <is>
           <t>Открытые двери и экскурсии</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="11">
-      <c r="A17" s="24" t="inlineStr">
+      <c r="A17" s="26" t="inlineStr">
         <is>
           <t>Категория</t>
         </is>
       </c>
-      <c r="B17" s="24" t="inlineStr">
+      <c r="B17" s="26" t="inlineStr">
         <is>
           <t>Природа и загородные поездки</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="11">
-      <c r="A18" s="24" t="inlineStr">
+      <c r="A18" s="26" t="inlineStr">
         <is>
           <t>Категория</t>
         </is>
       </c>
-      <c r="B18" s="24" t="inlineStr">
+      <c r="B18" s="26" t="inlineStr">
         <is>
           <t>Праздники и сезонное</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="11">
-      <c r="A19" s="24" t="inlineStr">
+      <c r="A19" s="26" t="inlineStr">
         <is>
           <t>Категория</t>
         </is>
       </c>
-      <c r="B19" s="24" t="inlineStr">
+      <c r="B19" s="26" t="inlineStr">
         <is>
           <t>Воркшопы и курсы</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="11">
-      <c r="A20" s="24" t="inlineStr">
+      <c r="A20" s="26" t="inlineStr">
         <is>
           <t>Категория</t>
         </is>
       </c>
-      <c r="B20" s="24" t="inlineStr">
+      <c r="B20" s="26" t="inlineStr">
         <is>
           <t>Сообщества и благотворительность</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="11">
-      <c r="A21" s="24" t="inlineStr">
+      <c r="A21" s="26" t="inlineStr">
         <is>
           <t>Категория</t>
         </is>
       </c>
-      <c r="B21" s="24" t="inlineStr">
+      <c r="B21" s="26" t="inlineStr">
         <is>
           <t>Практическое</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="11">
-      <c r="A22" s="24" t="inlineStr">
+      <c r="A22" s="26" t="inlineStr">
         <is>
           <t>Аудитория</t>
         </is>
       </c>
-      <c r="B22" s="24" t="inlineStr">
+      <c r="B22" s="26" t="inlineStr">
         <is>
           <t>дети до 5</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="11">
-      <c r="A23" s="24" t="inlineStr">
+      <c r="A23" s="26" t="inlineStr">
         <is>
           <t>Аудитория</t>
         </is>
       </c>
-      <c r="B23" s="24" t="inlineStr">
+      <c r="B23" s="26" t="inlineStr">
         <is>
           <t>дети 5–12</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="11">
-      <c r="A24" s="24" t="inlineStr">
+      <c r="A24" s="26" t="inlineStr">
         <is>
           <t>Аудитория</t>
         </is>
       </c>
-      <c r="B24" s="24" t="inlineStr">
+      <c r="B24" s="26" t="inlineStr">
         <is>
           <t>подростки</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="11">
-      <c r="A25" s="24" t="inlineStr">
+      <c r="A25" s="26" t="inlineStr">
         <is>
           <t>Аудитория</t>
         </is>
       </c>
-      <c r="B25" s="24" t="inlineStr">
+      <c r="B25" s="26" t="inlineStr">
         <is>
           <t>семьи</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="11">
-      <c r="A26" s="24" t="inlineStr">
+      <c r="A26" s="26" t="inlineStr">
         <is>
           <t>Аудитория</t>
         </is>
       </c>
-      <c r="B26" s="24" t="inlineStr">
+      <c r="B26" s="26" t="inlineStr">
         <is>
           <t>18+</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="11">
-      <c r="A27" s="24" t="inlineStr">
+      <c r="A27" s="26" t="inlineStr">
         <is>
           <t>Цена</t>
         </is>
       </c>
-      <c r="B27" s="24" t="inlineStr">
+      <c r="B27" s="26" t="inlineStr">
         <is>
           <t>бесплатно</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="11">
-      <c r="A28" s="24" t="inlineStr">
+      <c r="A28" s="26" t="inlineStr">
         <is>
           <t>Цена</t>
         </is>
       </c>
-      <c r="B28" s="24" t="inlineStr">
+      <c r="B28" s="26" t="inlineStr">
         <is>
           <t>до £10</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="11">
-      <c r="A29" s="24" t="inlineStr">
+      <c r="A29" s="26" t="inlineStr">
         <is>
           <t>Цена</t>
         </is>
       </c>
-      <c r="B29" s="24" t="inlineStr">
+      <c r="B29" s="26" t="inlineStr">
         <is>
           <t>дороже</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="11">
-      <c r="A30" s="24" t="inlineStr">
+      <c r="A30" s="26" t="inlineStr">
         <is>
           <t>Зона</t>
         </is>
       </c>
-      <c r="B30" s="24" t="inlineStr">
+      <c r="B30" s="26" t="inlineStr">
         <is>
           <t>Центр</t>
         </is>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="11">
-      <c r="A31" s="24" t="inlineStr">
+      <c r="A31" s="26" t="inlineStr">
         <is>
           <t>Зона</t>
         </is>
       </c>
-      <c r="B31" s="24" t="inlineStr">
+      <c r="B31" s="26" t="inlineStr">
         <is>
           <t>до 30 мин</t>
         </is>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="11">
-      <c r="A32" s="24" t="inlineStr">
+      <c r="A32" s="26" t="inlineStr">
         <is>
           <t>Зона</t>
         </is>
       </c>
-      <c r="B32" s="24" t="inlineStr">
+      <c r="B32" s="26" t="inlineStr">
         <is>
           <t>до часа</t>
         </is>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="11">
-      <c r="A33" s="24" t="inlineStr">
+      <c r="A33" s="26" t="inlineStr">
         <is>
           <t>Бронирование</t>
         </is>
       </c>
-      <c r="B33" s="24" t="inlineStr">
+      <c r="B33" s="26" t="inlineStr">
         <is>
           <t>без билетов</t>
         </is>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="11">
-      <c r="A34" s="24" t="inlineStr">
+      <c r="A34" s="26" t="inlineStr">
         <is>
           <t>Бронирование</t>
         </is>
       </c>
-      <c r="B34" s="24" t="inlineStr">
+      <c r="B34" s="26" t="inlineStr">
         <is>
           <t>нужно бронировать</t>
         </is>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="11">
-      <c r="A35" s="24" t="inlineStr">
+      <c r="A35" s="26" t="inlineStr">
         <is>
           <t>Бронирование</t>
         </is>
       </c>
-      <c r="B35" s="24" t="inlineStr">
+      <c r="B35" s="26" t="inlineStr">
         <is>
           <t>продажа открывается скоро</t>
         </is>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="11">
-      <c r="A36" s="24" t="inlineStr">
+      <c r="A36" s="26" t="inlineStr">
         <is>
           <t>Статус</t>
         </is>
       </c>
-      <c r="B36" s="24" t="inlineStr">
+      <c r="B36" s="26" t="inlineStr">
         <is>
           <t>по плану</t>
         </is>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="11">
-      <c r="A37" s="24" t="inlineStr">
+      <c r="A37" s="26" t="inlineStr">
         <is>
           <t>Статус</t>
         </is>
       </c>
-      <c r="B37" s="24" t="inlineStr">
+      <c r="B37" s="26" t="inlineStr">
         <is>
           <t>перенесено</t>
         </is>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="11">
-      <c r="A38" s="24" t="inlineStr">
+      <c r="A38" s="26" t="inlineStr">
         <is>
           <t>Статус</t>
         </is>
       </c>
-      <c r="B38" s="24" t="inlineStr">
+      <c r="B38" s="26" t="inlineStr">
         <is>
           <t>отменено</t>
         </is>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="11">
-      <c r="A39" s="24" t="inlineStr">
+      <c r="A39" s="26" t="inlineStr">
         <is>
           <t>Статус</t>
         </is>
       </c>
-      <c r="B39" s="24" t="inlineStr">
+      <c r="B39" s="26" t="inlineStr">
         <is>
           <t>sold out</t>
         </is>

</xml_diff>